<commit_message>
feat: update guardian phone numbers for all summer school students
</commit_message>
<xml_diff>
--- a/yazokulu.xlsx
+++ b/yazokulu.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\American Life S.tepe\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\American Life S.tepe\Documents\Codex\2026-07-09\can-you-see-or-access-my\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -6493,23 +6493,14 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6525,12 +6516,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6541,29 +6527,34 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6575,10 +6566,10 @@
     <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="25" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6590,22 +6581,25 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6626,12 +6620,6 @@
     <xf numFmtId="0" fontId="33" fillId="27" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="37" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6641,29 +6629,20 @@
     <xf numFmtId="0" fontId="4" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6671,8 +6650,29 @@
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6924,33 +6924,33 @@
       <c r="A1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="400" t="s">
+      <c r="B1" s="395" t="s">
         <v>219</v>
       </c>
-      <c r="C1" s="391"/>
-      <c r="D1" s="391"/>
-      <c r="E1" s="391"/>
-      <c r="F1" s="391"/>
-      <c r="G1" s="391"/>
-      <c r="H1" s="391"/>
-      <c r="I1" s="391"/>
-      <c r="J1" s="391"/>
-      <c r="K1" s="391"/>
-      <c r="L1" s="392"/>
+      <c r="C1" s="392"/>
+      <c r="D1" s="392"/>
+      <c r="E1" s="392"/>
+      <c r="F1" s="392"/>
+      <c r="G1" s="392"/>
+      <c r="H1" s="392"/>
+      <c r="I1" s="392"/>
+      <c r="J1" s="392"/>
+      <c r="K1" s="392"/>
+      <c r="L1" s="393"/>
     </row>
     <row r="2" spans="1:13" ht="27.75" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="401"/>
-      <c r="C2" s="391"/>
-      <c r="D2" s="391"/>
-      <c r="E2" s="391"/>
-      <c r="F2" s="391"/>
-      <c r="G2" s="391"/>
-      <c r="H2" s="391"/>
-      <c r="I2" s="391"/>
-      <c r="J2" s="391"/>
-      <c r="K2" s="391"/>
-      <c r="L2" s="392"/>
+      <c r="B2" s="396"/>
+      <c r="C2" s="392"/>
+      <c r="D2" s="392"/>
+      <c r="E2" s="392"/>
+      <c r="F2" s="392"/>
+      <c r="G2" s="392"/>
+      <c r="H2" s="392"/>
+      <c r="I2" s="392"/>
+      <c r="J2" s="392"/>
+      <c r="K2" s="392"/>
+      <c r="L2" s="393"/>
     </row>
     <row r="3" spans="1:13" ht="14.4">
       <c r="A3" s="2"/>
@@ -8026,19 +8026,19 @@
     </row>
     <row r="34" spans="1:25" ht="15.75" customHeight="1">
       <c r="A34" s="33"/>
-      <c r="B34" s="402" t="s">
+      <c r="B34" s="397" t="s">
         <v>242</v>
       </c>
-      <c r="C34" s="391"/>
-      <c r="D34" s="391"/>
-      <c r="E34" s="391"/>
-      <c r="F34" s="391"/>
-      <c r="G34" s="391"/>
-      <c r="H34" s="391"/>
-      <c r="I34" s="391"/>
-      <c r="J34" s="391"/>
-      <c r="K34" s="391"/>
-      <c r="L34" s="392"/>
+      <c r="C34" s="392"/>
+      <c r="D34" s="392"/>
+      <c r="E34" s="392"/>
+      <c r="F34" s="392"/>
+      <c r="G34" s="392"/>
+      <c r="H34" s="392"/>
+      <c r="I34" s="392"/>
+      <c r="J34" s="392"/>
+      <c r="K34" s="392"/>
+      <c r="L34" s="393"/>
       <c r="M34" s="35"/>
       <c r="N34" s="35"/>
       <c r="O34" s="35"/>
@@ -8611,19 +8611,19 @@
     </row>
     <row r="51" spans="1:16" ht="20.25" customHeight="1">
       <c r="A51" s="2"/>
-      <c r="B51" s="403" t="s">
+      <c r="B51" s="398" t="s">
         <v>257</v>
       </c>
-      <c r="C51" s="391"/>
-      <c r="D51" s="391"/>
-      <c r="E51" s="391"/>
-      <c r="F51" s="391"/>
-      <c r="G51" s="391"/>
-      <c r="H51" s="391"/>
-      <c r="I51" s="391"/>
-      <c r="J51" s="391"/>
-      <c r="K51" s="391"/>
-      <c r="L51" s="392"/>
+      <c r="C51" s="392"/>
+      <c r="D51" s="392"/>
+      <c r="E51" s="392"/>
+      <c r="F51" s="392"/>
+      <c r="G51" s="392"/>
+      <c r="H51" s="392"/>
+      <c r="I51" s="392"/>
+      <c r="J51" s="392"/>
+      <c r="K51" s="392"/>
+      <c r="L51" s="393"/>
     </row>
     <row r="52" spans="1:16" ht="20.25" customHeight="1">
       <c r="A52" s="2"/>
@@ -9200,9 +9200,9 @@
       <c r="E71" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F71" s="404"/>
-      <c r="G71" s="395"/>
-      <c r="H71" s="395"/>
+      <c r="F71" s="399"/>
+      <c r="G71" s="400"/>
+      <c r="H71" s="400"/>
       <c r="J71" s="87"/>
     </row>
     <row r="72" spans="1:12" ht="15.75" customHeight="1">
@@ -9359,19 +9359,19 @@
     </row>
     <row r="82" spans="1:25" ht="21">
       <c r="A82" s="2"/>
-      <c r="B82" s="405" t="s">
+      <c r="B82" s="391" t="s">
         <v>263</v>
       </c>
-      <c r="C82" s="391"/>
-      <c r="D82" s="391"/>
-      <c r="E82" s="391"/>
-      <c r="F82" s="391"/>
-      <c r="G82" s="391"/>
-      <c r="H82" s="391"/>
-      <c r="I82" s="391"/>
-      <c r="J82" s="391"/>
-      <c r="K82" s="391"/>
-      <c r="L82" s="392"/>
+      <c r="C82" s="392"/>
+      <c r="D82" s="392"/>
+      <c r="E82" s="392"/>
+      <c r="F82" s="392"/>
+      <c r="G82" s="392"/>
+      <c r="H82" s="392"/>
+      <c r="I82" s="392"/>
+      <c r="J82" s="392"/>
+      <c r="K82" s="392"/>
+      <c r="L82" s="393"/>
     </row>
     <row r="83" spans="1:25" ht="15.75" customHeight="1">
       <c r="A83" s="2"/>
@@ -10356,19 +10356,19 @@
     </row>
     <row r="113" spans="1:13" ht="21">
       <c r="A113" s="2"/>
-      <c r="B113" s="406" t="s">
+      <c r="B113" s="394" t="s">
         <v>275</v>
       </c>
-      <c r="C113" s="391"/>
-      <c r="D113" s="391"/>
-      <c r="E113" s="391"/>
-      <c r="F113" s="391"/>
-      <c r="G113" s="391"/>
-      <c r="H113" s="391"/>
-      <c r="I113" s="391"/>
-      <c r="J113" s="391"/>
-      <c r="K113" s="391"/>
-      <c r="L113" s="392"/>
+      <c r="C113" s="392"/>
+      <c r="D113" s="392"/>
+      <c r="E113" s="392"/>
+      <c r="F113" s="392"/>
+      <c r="G113" s="392"/>
+      <c r="H113" s="392"/>
+      <c r="I113" s="392"/>
+      <c r="J113" s="392"/>
+      <c r="K113" s="392"/>
+      <c r="L113" s="393"/>
     </row>
     <row r="114" spans="1:13" ht="15.75" customHeight="1">
       <c r="A114" s="2"/>
@@ -22495,37 +22495,37 @@
       <c r="A2" s="458" t="s">
         <v>988</v>
       </c>
-      <c r="B2" s="410"/>
-      <c r="C2" s="410"/>
-      <c r="D2" s="410"/>
-      <c r="E2" s="410"/>
-      <c r="F2" s="410"/>
-      <c r="G2" s="410"/>
-      <c r="H2" s="410"/>
-      <c r="I2" s="410"/>
-      <c r="J2" s="410"/>
-      <c r="K2" s="410"/>
-      <c r="L2" s="410"/>
-      <c r="M2" s="410"/>
-      <c r="N2" s="410"/>
-      <c r="O2" s="411"/>
+      <c r="B2" s="404"/>
+      <c r="C2" s="404"/>
+      <c r="D2" s="404"/>
+      <c r="E2" s="404"/>
+      <c r="F2" s="404"/>
+      <c r="G2" s="404"/>
+      <c r="H2" s="404"/>
+      <c r="I2" s="404"/>
+      <c r="J2" s="404"/>
+      <c r="K2" s="404"/>
+      <c r="L2" s="404"/>
+      <c r="M2" s="404"/>
+      <c r="N2" s="404"/>
+      <c r="O2" s="405"/>
     </row>
     <row r="3" spans="1:16">
-      <c r="A3" s="412"/>
-      <c r="B3" s="398"/>
-      <c r="C3" s="398"/>
-      <c r="D3" s="398"/>
-      <c r="E3" s="398"/>
-      <c r="F3" s="398"/>
-      <c r="G3" s="398"/>
-      <c r="H3" s="398"/>
-      <c r="I3" s="398"/>
-      <c r="J3" s="398"/>
-      <c r="K3" s="398"/>
-      <c r="L3" s="398"/>
-      <c r="M3" s="398"/>
-      <c r="N3" s="398"/>
-      <c r="O3" s="399"/>
+      <c r="A3" s="406"/>
+      <c r="B3" s="407"/>
+      <c r="C3" s="407"/>
+      <c r="D3" s="407"/>
+      <c r="E3" s="407"/>
+      <c r="F3" s="407"/>
+      <c r="G3" s="407"/>
+      <c r="H3" s="407"/>
+      <c r="I3" s="407"/>
+      <c r="J3" s="407"/>
+      <c r="K3" s="407"/>
+      <c r="L3" s="407"/>
+      <c r="M3" s="407"/>
+      <c r="N3" s="407"/>
+      <c r="O3" s="408"/>
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="362"/>
@@ -22533,7 +22533,7 @@
         <v>989</v>
       </c>
       <c r="C4" s="363"/>
-      <c r="D4" s="394" t="s">
+      <c r="D4" s="457" t="s">
         <v>990</v>
       </c>
       <c r="E4" s="2"/>
@@ -22542,7 +22542,7 @@
         <v>991</v>
       </c>
       <c r="H4" s="363"/>
-      <c r="I4" s="394" t="s">
+      <c r="I4" s="457" t="s">
         <v>990</v>
       </c>
       <c r="K4" s="364"/>
@@ -22550,7 +22550,7 @@
         <v>992</v>
       </c>
       <c r="M4" s="364"/>
-      <c r="N4" s="394" t="s">
+      <c r="N4" s="457" t="s">
         <v>990</v>
       </c>
     </row>
@@ -22562,7 +22562,7 @@
       <c r="C5" s="362" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="395"/>
+      <c r="D5" s="400"/>
       <c r="E5" s="2"/>
       <c r="F5" s="362"/>
       <c r="G5" s="362" t="s">
@@ -22571,7 +22571,7 @@
       <c r="H5" s="362" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="395"/>
+      <c r="I5" s="400"/>
       <c r="K5" s="362"/>
       <c r="L5" s="362" t="s">
         <v>7</v>
@@ -22579,7 +22579,7 @@
       <c r="M5" s="362" t="s">
         <v>8</v>
       </c>
-      <c r="N5" s="395"/>
+      <c r="N5" s="400"/>
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="10">
@@ -23132,20 +23132,20 @@
       <c r="A19" s="459" t="s">
         <v>1027</v>
       </c>
-      <c r="B19" s="410"/>
-      <c r="C19" s="410"/>
-      <c r="D19" s="410"/>
-      <c r="E19" s="410"/>
-      <c r="F19" s="410"/>
-      <c r="G19" s="410"/>
-      <c r="H19" s="410"/>
-      <c r="I19" s="410"/>
-      <c r="J19" s="410"/>
-      <c r="K19" s="410"/>
-      <c r="L19" s="410"/>
-      <c r="M19" s="410"/>
-      <c r="N19" s="410"/>
-      <c r="O19" s="411"/>
+      <c r="B19" s="404"/>
+      <c r="C19" s="404"/>
+      <c r="D19" s="404"/>
+      <c r="E19" s="404"/>
+      <c r="F19" s="404"/>
+      <c r="G19" s="404"/>
+      <c r="H19" s="404"/>
+      <c r="I19" s="404"/>
+      <c r="J19" s="404"/>
+      <c r="K19" s="404"/>
+      <c r="L19" s="404"/>
+      <c r="M19" s="404"/>
+      <c r="N19" s="404"/>
+      <c r="O19" s="405"/>
       <c r="P19" s="35"/>
       <c r="Q19" s="35"/>
       <c r="R19" s="35"/>
@@ -23156,21 +23156,21 @@
       <c r="W19" s="35"/>
     </row>
     <row r="20" spans="1:23">
-      <c r="A20" s="412"/>
-      <c r="B20" s="398"/>
-      <c r="C20" s="398"/>
-      <c r="D20" s="398"/>
-      <c r="E20" s="398"/>
-      <c r="F20" s="398"/>
-      <c r="G20" s="398"/>
-      <c r="H20" s="398"/>
-      <c r="I20" s="398"/>
-      <c r="J20" s="398"/>
-      <c r="K20" s="398"/>
-      <c r="L20" s="398"/>
-      <c r="M20" s="398"/>
-      <c r="N20" s="398"/>
-      <c r="O20" s="399"/>
+      <c r="A20" s="406"/>
+      <c r="B20" s="407"/>
+      <c r="C20" s="407"/>
+      <c r="D20" s="407"/>
+      <c r="E20" s="407"/>
+      <c r="F20" s="407"/>
+      <c r="G20" s="407"/>
+      <c r="H20" s="407"/>
+      <c r="I20" s="407"/>
+      <c r="J20" s="407"/>
+      <c r="K20" s="407"/>
+      <c r="L20" s="407"/>
+      <c r="M20" s="407"/>
+      <c r="N20" s="407"/>
+      <c r="O20" s="408"/>
       <c r="P20" s="35"/>
       <c r="Q20" s="35"/>
       <c r="R20" s="35"/>
@@ -23186,7 +23186,7 @@
         <v>989</v>
       </c>
       <c r="C21" s="382"/>
-      <c r="D21" s="394" t="s">
+      <c r="D21" s="457" t="s">
         <v>990</v>
       </c>
       <c r="E21" s="2"/>
@@ -23195,7 +23195,7 @@
         <v>991</v>
       </c>
       <c r="H21" s="383"/>
-      <c r="I21" s="394" t="s">
+      <c r="I21" s="457" t="s">
         <v>990</v>
       </c>
       <c r="K21" s="362"/>
@@ -23203,7 +23203,7 @@
         <v>992</v>
       </c>
       <c r="M21" s="364"/>
-      <c r="N21" s="394" t="s">
+      <c r="N21" s="457" t="s">
         <v>990</v>
       </c>
     </row>
@@ -23215,7 +23215,7 @@
       <c r="C22" s="362" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="395"/>
+      <c r="D22" s="400"/>
       <c r="E22" s="2"/>
       <c r="F22" s="362"/>
       <c r="G22" s="362" t="s">
@@ -23224,7 +23224,7 @@
       <c r="H22" s="362" t="s">
         <v>8</v>
       </c>
-      <c r="I22" s="395"/>
+      <c r="I22" s="400"/>
       <c r="K22" s="364"/>
       <c r="L22" s="362" t="s">
         <v>7</v>
@@ -23232,7 +23232,7 @@
       <c r="M22" s="362" t="s">
         <v>8</v>
       </c>
-      <c r="N22" s="395"/>
+      <c r="N22" s="400"/>
     </row>
     <row r="23" spans="1:23">
       <c r="A23" s="10">
@@ -28608,52 +28608,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="100.5" customHeight="1">
-      <c r="A1" s="409" t="s">
+      <c r="A1" s="403" t="s">
         <v>290</v>
       </c>
-      <c r="B1" s="410"/>
-      <c r="C1" s="410"/>
-      <c r="D1" s="410"/>
-      <c r="E1" s="410"/>
-      <c r="F1" s="410"/>
-      <c r="G1" s="410"/>
-      <c r="H1" s="410"/>
-      <c r="I1" s="410"/>
-      <c r="J1" s="410"/>
-      <c r="K1" s="410"/>
-      <c r="L1" s="410"/>
-      <c r="M1" s="411"/>
+      <c r="B1" s="404"/>
+      <c r="C1" s="404"/>
+      <c r="D1" s="404"/>
+      <c r="E1" s="404"/>
+      <c r="F1" s="404"/>
+      <c r="G1" s="404"/>
+      <c r="H1" s="404"/>
+      <c r="I1" s="404"/>
+      <c r="J1" s="404"/>
+      <c r="K1" s="404"/>
+      <c r="L1" s="404"/>
+      <c r="M1" s="405"/>
     </row>
     <row r="2" spans="1:13" ht="1.5" customHeight="1">
-      <c r="A2" s="412"/>
-      <c r="B2" s="398"/>
-      <c r="C2" s="398"/>
-      <c r="D2" s="398"/>
-      <c r="E2" s="398"/>
-      <c r="F2" s="398"/>
-      <c r="G2" s="398"/>
-      <c r="H2" s="398"/>
-      <c r="I2" s="398"/>
-      <c r="J2" s="398"/>
-      <c r="K2" s="398"/>
-      <c r="L2" s="398"/>
-      <c r="M2" s="399"/>
+      <c r="A2" s="406"/>
+      <c r="B2" s="407"/>
+      <c r="C2" s="407"/>
+      <c r="D2" s="407"/>
+      <c r="E2" s="407"/>
+      <c r="F2" s="407"/>
+      <c r="G2" s="407"/>
+      <c r="H2" s="407"/>
+      <c r="I2" s="407"/>
+      <c r="J2" s="407"/>
+      <c r="K2" s="407"/>
+      <c r="L2" s="407"/>
+      <c r="M2" s="408"/>
     </row>
     <row r="3" spans="1:13" ht="38.25" customHeight="1">
-      <c r="A3" s="393" t="s">
+      <c r="A3" s="409" t="s">
         <v>291</v>
       </c>
-      <c r="B3" s="391"/>
-      <c r="C3" s="391"/>
-      <c r="D3" s="391"/>
-      <c r="E3" s="391"/>
-      <c r="F3" s="391"/>
-      <c r="G3" s="391"/>
-      <c r="H3" s="391"/>
-      <c r="I3" s="391"/>
-      <c r="J3" s="391"/>
-      <c r="K3" s="391"/>
-      <c r="L3" s="392"/>
+      <c r="B3" s="392"/>
+      <c r="C3" s="392"/>
+      <c r="D3" s="392"/>
+      <c r="E3" s="392"/>
+      <c r="F3" s="392"/>
+      <c r="G3" s="392"/>
+      <c r="H3" s="392"/>
+      <c r="I3" s="392"/>
+      <c r="J3" s="392"/>
+      <c r="K3" s="392"/>
+      <c r="L3" s="393"/>
     </row>
     <row r="4" spans="1:13" ht="14.4">
       <c r="A4" s="179" t="s">
@@ -29469,19 +29469,19 @@
       <c r="P34" s="35"/>
     </row>
     <row r="35" spans="1:16" ht="26.25" customHeight="1">
-      <c r="A35" s="396" t="s">
+      <c r="A35" s="410" t="s">
         <v>297</v>
       </c>
-      <c r="B35" s="391"/>
-      <c r="C35" s="391"/>
-      <c r="D35" s="391"/>
-      <c r="E35" s="391"/>
-      <c r="F35" s="391"/>
-      <c r="G35" s="391"/>
-      <c r="H35" s="391"/>
-      <c r="I35" s="391"/>
-      <c r="J35" s="391"/>
-      <c r="K35" s="392"/>
+      <c r="B35" s="392"/>
+      <c r="C35" s="392"/>
+      <c r="D35" s="392"/>
+      <c r="E35" s="392"/>
+      <c r="F35" s="392"/>
+      <c r="G35" s="392"/>
+      <c r="H35" s="392"/>
+      <c r="I35" s="392"/>
+      <c r="J35" s="392"/>
+      <c r="K35" s="393"/>
       <c r="L35" s="35"/>
       <c r="M35" s="35"/>
       <c r="N35" s="35"/>
@@ -29909,19 +29909,19 @@
       <c r="O50" s="32"/>
     </row>
     <row r="52" spans="1:15" ht="21">
-      <c r="A52" s="403" t="s">
+      <c r="A52" s="398" t="s">
         <v>299</v>
       </c>
-      <c r="B52" s="391"/>
-      <c r="C52" s="391"/>
-      <c r="D52" s="391"/>
-      <c r="E52" s="391"/>
-      <c r="F52" s="391"/>
-      <c r="G52" s="391"/>
-      <c r="H52" s="391"/>
-      <c r="I52" s="391"/>
-      <c r="J52" s="391"/>
-      <c r="K52" s="392"/>
+      <c r="B52" s="392"/>
+      <c r="C52" s="392"/>
+      <c r="D52" s="392"/>
+      <c r="E52" s="392"/>
+      <c r="F52" s="392"/>
+      <c r="G52" s="392"/>
+      <c r="H52" s="392"/>
+      <c r="I52" s="392"/>
+      <c r="J52" s="392"/>
+      <c r="K52" s="393"/>
     </row>
     <row r="53" spans="1:15" ht="20.25" customHeight="1">
       <c r="A53" s="195" t="s">
@@ -30373,9 +30373,9 @@
       <c r="B72" s="199"/>
       <c r="C72" s="17"/>
       <c r="D72" s="89"/>
-      <c r="E72" s="404"/>
-      <c r="F72" s="395"/>
-      <c r="G72" s="395"/>
+      <c r="E72" s="399"/>
+      <c r="F72" s="400"/>
+      <c r="G72" s="400"/>
       <c r="I72" s="87"/>
     </row>
     <row r="73" spans="1:11" ht="14.4">
@@ -30497,19 +30497,19 @@
       <c r="P82" s="96"/>
     </row>
     <row r="83" spans="1:16" ht="21">
-      <c r="A83" s="405" t="s">
+      <c r="A83" s="391" t="s">
         <v>300</v>
       </c>
-      <c r="B83" s="391"/>
-      <c r="C83" s="391"/>
-      <c r="D83" s="391"/>
-      <c r="E83" s="391"/>
-      <c r="F83" s="391"/>
-      <c r="G83" s="391"/>
-      <c r="H83" s="391"/>
-      <c r="I83" s="391"/>
-      <c r="J83" s="391"/>
-      <c r="K83" s="392"/>
+      <c r="B83" s="392"/>
+      <c r="C83" s="392"/>
+      <c r="D83" s="392"/>
+      <c r="E83" s="392"/>
+      <c r="F83" s="392"/>
+      <c r="G83" s="392"/>
+      <c r="H83" s="392"/>
+      <c r="I83" s="392"/>
+      <c r="J83" s="392"/>
+      <c r="K83" s="393"/>
       <c r="L83" s="200"/>
     </row>
     <row r="84" spans="1:16" ht="14.4">
@@ -31277,34 +31277,34 @@
       <c r="H113" s="2"/>
     </row>
     <row r="114" spans="1:12" ht="21">
-      <c r="A114" s="406" t="s">
+      <c r="A114" s="394" t="s">
         <v>302</v>
       </c>
-      <c r="B114" s="391"/>
-      <c r="C114" s="391"/>
-      <c r="D114" s="391"/>
-      <c r="E114" s="391"/>
-      <c r="F114" s="391"/>
-      <c r="G114" s="391"/>
-      <c r="H114" s="391"/>
-      <c r="I114" s="391"/>
-      <c r="J114" s="391"/>
-      <c r="K114" s="392"/>
+      <c r="B114" s="392"/>
+      <c r="C114" s="392"/>
+      <c r="D114" s="392"/>
+      <c r="E114" s="392"/>
+      <c r="F114" s="392"/>
+      <c r="G114" s="392"/>
+      <c r="H114" s="392"/>
+      <c r="I114" s="392"/>
+      <c r="J114" s="392"/>
+      <c r="K114" s="393"/>
     </row>
     <row r="115" spans="1:12" ht="14.4">
-      <c r="A115" s="407" t="s">
+      <c r="A115" s="401" t="s">
         <v>68</v>
       </c>
       <c r="B115" s="168"/>
       <c r="C115" s="168"/>
       <c r="D115" s="120"/>
-      <c r="E115" s="407" t="s">
+      <c r="E115" s="401" t="s">
         <v>135</v>
       </c>
       <c r="F115" s="168"/>
       <c r="G115" s="168"/>
       <c r="H115" s="120"/>
-      <c r="I115" s="407" t="s">
+      <c r="I115" s="401" t="s">
         <v>5</v>
       </c>
       <c r="J115" s="168"/>
@@ -31312,7 +31312,7 @@
       <c r="L115" s="120"/>
     </row>
     <row r="116" spans="1:12" ht="58.5" customHeight="1">
-      <c r="A116" s="408"/>
+      <c r="A116" s="402"/>
       <c r="B116" s="169" t="s">
         <v>7</v>
       </c>
@@ -31322,7 +31322,7 @@
       <c r="D116" s="160" t="s">
         <v>292</v>
       </c>
-      <c r="E116" s="408"/>
+      <c r="E116" s="402"/>
       <c r="F116" s="169" t="s">
         <v>7</v>
       </c>
@@ -31332,7 +31332,7 @@
       <c r="H116" s="160" t="s">
         <v>292</v>
       </c>
-      <c r="I116" s="408"/>
+      <c r="I116" s="402"/>
       <c r="J116" s="169" t="s">
         <v>7</v>
       </c>
@@ -31673,7 +31673,7 @@
       <c r="L130" s="35"/>
     </row>
     <row r="131" spans="1:12" ht="14.4">
-      <c r="A131" s="407" t="s">
+      <c r="A131" s="401" t="s">
         <v>3</v>
       </c>
       <c r="B131" s="168"/>
@@ -31688,7 +31688,7 @@
       <c r="K131" s="2"/>
     </row>
     <row r="132" spans="1:12" ht="57" customHeight="1">
-      <c r="A132" s="408"/>
+      <c r="A132" s="402"/>
       <c r="B132" s="169" t="s">
         <v>7</v>
       </c>
@@ -32576,124 +32576,124 @@
   <sheetData>
     <row r="1" spans="1:17" ht="100.5" customHeight="1">
       <c r="A1" s="210"/>
-      <c r="B1" s="419" t="s">
+      <c r="B1" s="429" t="s">
         <v>326</v>
       </c>
-      <c r="C1" s="391"/>
-      <c r="D1" s="391"/>
-      <c r="E1" s="391"/>
-      <c r="F1" s="391"/>
-      <c r="G1" s="391"/>
-      <c r="H1" s="391"/>
-      <c r="I1" s="391"/>
-      <c r="J1" s="391"/>
-      <c r="K1" s="391"/>
-      <c r="L1" s="391"/>
-      <c r="M1" s="391"/>
-      <c r="N1" s="392"/>
+      <c r="C1" s="392"/>
+      <c r="D1" s="392"/>
+      <c r="E1" s="392"/>
+      <c r="F1" s="392"/>
+      <c r="G1" s="392"/>
+      <c r="H1" s="392"/>
+      <c r="I1" s="392"/>
+      <c r="J1" s="392"/>
+      <c r="K1" s="392"/>
+      <c r="L1" s="392"/>
+      <c r="M1" s="392"/>
+      <c r="N1" s="393"/>
       <c r="Q1" s="35"/>
     </row>
     <row r="2" spans="1:17" ht="38.25" customHeight="1">
       <c r="A2" s="211"/>
-      <c r="B2" s="420" t="s">
+      <c r="B2" s="430" t="s">
         <v>291</v>
       </c>
-      <c r="C2" s="391"/>
-      <c r="D2" s="391"/>
-      <c r="E2" s="391"/>
-      <c r="F2" s="391"/>
-      <c r="G2" s="391"/>
-      <c r="H2" s="391"/>
-      <c r="I2" s="391"/>
-      <c r="J2" s="391"/>
-      <c r="K2" s="391"/>
-      <c r="L2" s="391"/>
-      <c r="M2" s="391"/>
-      <c r="N2" s="392"/>
+      <c r="C2" s="392"/>
+      <c r="D2" s="392"/>
+      <c r="E2" s="392"/>
+      <c r="F2" s="392"/>
+      <c r="G2" s="392"/>
+      <c r="H2" s="392"/>
+      <c r="I2" s="392"/>
+      <c r="J2" s="392"/>
+      <c r="K2" s="392"/>
+      <c r="L2" s="392"/>
+      <c r="M2" s="392"/>
+      <c r="N2" s="393"/>
       <c r="Q2" s="35"/>
     </row>
     <row r="3" spans="1:17" ht="14.4">
       <c r="A3" s="34"/>
-      <c r="B3" s="421" t="s">
+      <c r="B3" s="422" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="179">
         <v>108</v>
       </c>
       <c r="D3" s="179"/>
-      <c r="E3" s="414" t="s">
+      <c r="E3" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="F3" s="421" t="s">
+      <c r="F3" s="422" t="s">
         <v>3</v>
       </c>
       <c r="G3" s="179">
         <v>105</v>
       </c>
       <c r="H3" s="179"/>
-      <c r="I3" s="414" t="s">
+      <c r="I3" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="J3" s="421" t="s">
+      <c r="J3" s="422" t="s">
         <v>5</v>
       </c>
       <c r="K3" s="179">
         <v>103</v>
       </c>
       <c r="L3" s="179"/>
-      <c r="M3" s="414" t="s">
+      <c r="M3" s="411" t="s">
         <v>327</v>
       </c>
       <c r="Q3" s="35"/>
     </row>
     <row r="4" spans="1:17" ht="14.4">
       <c r="A4" s="34"/>
-      <c r="B4" s="413"/>
+      <c r="B4" s="412"/>
       <c r="C4" s="179" t="s">
         <v>328</v>
       </c>
       <c r="D4" s="179"/>
-      <c r="E4" s="413"/>
-      <c r="F4" s="413"/>
+      <c r="E4" s="412"/>
+      <c r="F4" s="412"/>
       <c r="G4" s="179" t="s">
         <v>220</v>
       </c>
       <c r="H4" s="179"/>
-      <c r="I4" s="413"/>
-      <c r="J4" s="413"/>
+      <c r="I4" s="412"/>
+      <c r="J4" s="412"/>
       <c r="K4" s="179" t="s">
         <v>329</v>
       </c>
       <c r="L4" s="179"/>
-      <c r="M4" s="413"/>
+      <c r="M4" s="412"/>
       <c r="Q4" s="35"/>
     </row>
     <row r="5" spans="1:17" ht="22.5" customHeight="1">
       <c r="A5" s="34"/>
-      <c r="B5" s="408"/>
+      <c r="B5" s="402"/>
       <c r="C5" s="180" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="180" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="408"/>
-      <c r="F5" s="408"/>
+      <c r="E5" s="402"/>
+      <c r="F5" s="402"/>
       <c r="G5" s="180" t="s">
         <v>7</v>
       </c>
       <c r="H5" s="180" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="408"/>
-      <c r="J5" s="408"/>
+      <c r="I5" s="402"/>
+      <c r="J5" s="402"/>
       <c r="K5" s="180" t="s">
         <v>7</v>
       </c>
       <c r="L5" s="180" t="s">
         <v>8</v>
       </c>
-      <c r="M5" s="408"/>
+      <c r="M5" s="402"/>
       <c r="Q5" s="35"/>
     </row>
     <row r="6" spans="1:17" ht="14.4">
@@ -33113,30 +33113,30 @@
     </row>
     <row r="19" spans="1:17" ht="14.4">
       <c r="A19" s="34"/>
-      <c r="B19" s="421" t="s">
+      <c r="B19" s="422" t="s">
         <v>68</v>
       </c>
       <c r="C19" s="179">
         <v>107</v>
       </c>
       <c r="D19" s="179"/>
-      <c r="E19" s="414" t="s">
+      <c r="E19" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="F19" s="428" t="s">
+      <c r="F19" s="425" t="s">
         <v>68</v>
       </c>
       <c r="G19" s="216">
         <v>106</v>
       </c>
       <c r="H19" s="217"/>
-      <c r="I19" s="429" t="s">
+      <c r="I19" s="426" t="s">
         <v>327</v>
       </c>
-      <c r="J19" s="430"/>
-      <c r="K19" s="431"/>
-      <c r="L19" s="395"/>
-      <c r="M19" s="422"/>
+      <c r="J19" s="416"/>
+      <c r="K19" s="427"/>
+      <c r="L19" s="400"/>
+      <c r="M19" s="419"/>
       <c r="N19" s="35"/>
       <c r="O19" s="35"/>
       <c r="P19" s="35"/>
@@ -33144,48 +33144,48 @@
     </row>
     <row r="20" spans="1:17" ht="21.75" customHeight="1">
       <c r="A20" s="34"/>
-      <c r="B20" s="413"/>
+      <c r="B20" s="412"/>
       <c r="C20" s="179" t="s">
         <v>343</v>
       </c>
       <c r="D20" s="179"/>
-      <c r="E20" s="413"/>
-      <c r="F20" s="413"/>
+      <c r="E20" s="412"/>
+      <c r="F20" s="412"/>
       <c r="G20" s="218" t="s">
         <v>344</v>
       </c>
       <c r="H20" s="217"/>
-      <c r="I20" s="413"/>
-      <c r="J20" s="395"/>
-      <c r="K20" s="395"/>
-      <c r="L20" s="395"/>
-      <c r="M20" s="395"/>
+      <c r="I20" s="412"/>
+      <c r="J20" s="400"/>
+      <c r="K20" s="400"/>
+      <c r="L20" s="400"/>
+      <c r="M20" s="400"/>
       <c r="N20" s="35"/>
       <c r="O20" s="35"/>
       <c r="Q20" s="35"/>
     </row>
     <row r="21" spans="1:17" ht="30.75" customHeight="1">
       <c r="A21" s="34"/>
-      <c r="B21" s="408"/>
+      <c r="B21" s="402"/>
       <c r="C21" s="179" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="180" t="s">
         <v>8</v>
       </c>
-      <c r="E21" s="408"/>
-      <c r="F21" s="408"/>
+      <c r="E21" s="402"/>
+      <c r="F21" s="402"/>
       <c r="G21" s="219" t="s">
         <v>7</v>
       </c>
       <c r="H21" s="219" t="s">
         <v>8</v>
       </c>
-      <c r="I21" s="408"/>
-      <c r="J21" s="395"/>
+      <c r="I21" s="402"/>
+      <c r="J21" s="400"/>
       <c r="K21" s="39"/>
       <c r="L21" s="39"/>
-      <c r="M21" s="395"/>
+      <c r="M21" s="400"/>
       <c r="N21" s="35"/>
       <c r="O21" s="35"/>
       <c r="Q21" s="35"/>
@@ -33221,7 +33221,7 @@
       <c r="L22" s="48"/>
       <c r="M22" s="9"/>
       <c r="N22" s="224"/>
-      <c r="O22" s="423"/>
+      <c r="O22" s="420"/>
       <c r="Q22" s="35"/>
     </row>
     <row r="23" spans="1:17" ht="14.4">
@@ -33255,7 +33255,7 @@
       <c r="L23" s="223"/>
       <c r="M23" s="89"/>
       <c r="N23" s="35"/>
-      <c r="O23" s="395"/>
+      <c r="O23" s="400"/>
       <c r="Q23" s="35"/>
     </row>
     <row r="24" spans="1:17" ht="14.4">
@@ -33289,7 +33289,7 @@
       <c r="L24" s="226"/>
       <c r="M24" s="35"/>
       <c r="N24" s="35"/>
-      <c r="O24" s="395"/>
+      <c r="O24" s="400"/>
       <c r="Q24" s="35"/>
     </row>
     <row r="25" spans="1:17" ht="14.4">
@@ -33323,7 +33323,7 @@
       <c r="L25" s="48"/>
       <c r="M25" s="89"/>
       <c r="N25" s="35"/>
-      <c r="O25" s="395"/>
+      <c r="O25" s="400"/>
       <c r="Q25" s="35"/>
     </row>
     <row r="26" spans="1:17" ht="14.4">
@@ -33560,19 +33560,19 @@
     </row>
     <row r="35" spans="1:17" ht="30.75" customHeight="1">
       <c r="A35" s="211"/>
-      <c r="B35" s="432" t="s">
+      <c r="B35" s="428" t="s">
         <v>297</v>
       </c>
-      <c r="C35" s="391"/>
-      <c r="D35" s="391"/>
-      <c r="E35" s="391"/>
-      <c r="F35" s="391"/>
-      <c r="G35" s="391"/>
-      <c r="H35" s="391"/>
-      <c r="I35" s="391"/>
-      <c r="J35" s="391"/>
-      <c r="K35" s="391"/>
-      <c r="L35" s="392"/>
+      <c r="C35" s="392"/>
+      <c r="D35" s="392"/>
+      <c r="E35" s="392"/>
+      <c r="F35" s="392"/>
+      <c r="G35" s="392"/>
+      <c r="H35" s="392"/>
+      <c r="I35" s="392"/>
+      <c r="J35" s="392"/>
+      <c r="K35" s="392"/>
+      <c r="L35" s="393"/>
       <c r="M35" s="35"/>
       <c r="N35" s="35"/>
       <c r="O35" s="35"/>
@@ -33581,24 +33581,24 @@
     </row>
     <row r="36" spans="1:17" ht="21.75" customHeight="1">
       <c r="A36" s="47"/>
-      <c r="B36" s="425" t="s">
+      <c r="B36" s="423" t="s">
         <v>0</v>
       </c>
       <c r="C36" s="231">
         <v>105</v>
       </c>
       <c r="D36" s="231"/>
-      <c r="E36" s="414" t="s">
+      <c r="E36" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="F36" s="433" t="s">
+      <c r="F36" s="415" t="s">
         <v>5</v>
       </c>
       <c r="G36" s="232">
         <v>107</v>
       </c>
       <c r="H36" s="231"/>
-      <c r="I36" s="414" t="s">
+      <c r="I36" s="411" t="s">
         <v>327</v>
       </c>
       <c r="J36" s="34"/>
@@ -33609,18 +33609,18 @@
     </row>
     <row r="37" spans="1:17" ht="21.75" customHeight="1">
       <c r="A37" s="47"/>
-      <c r="B37" s="413"/>
+      <c r="B37" s="412"/>
       <c r="C37" s="231" t="s">
         <v>352</v>
       </c>
       <c r="D37" s="231"/>
-      <c r="E37" s="413"/>
-      <c r="F37" s="413"/>
+      <c r="E37" s="412"/>
+      <c r="F37" s="412"/>
       <c r="G37" s="231" t="s">
         <v>343</v>
       </c>
       <c r="H37" s="231"/>
-      <c r="I37" s="413"/>
+      <c r="I37" s="412"/>
       <c r="J37" s="34"/>
       <c r="K37" s="34"/>
       <c r="L37" s="34"/>
@@ -33629,22 +33629,22 @@
     </row>
     <row r="38" spans="1:17" ht="30" customHeight="1">
       <c r="A38" s="47"/>
-      <c r="B38" s="408"/>
+      <c r="B38" s="402"/>
       <c r="C38" s="233" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="233" t="s">
         <v>8</v>
       </c>
-      <c r="E38" s="408"/>
-      <c r="F38" s="408"/>
+      <c r="E38" s="402"/>
+      <c r="F38" s="402"/>
       <c r="G38" s="233" t="s">
         <v>7</v>
       </c>
       <c r="H38" s="233" t="s">
         <v>8</v>
       </c>
-      <c r="I38" s="408"/>
+      <c r="I38" s="402"/>
       <c r="J38" s="34"/>
       <c r="K38" s="39"/>
       <c r="L38" s="39"/>
@@ -33676,9 +33676,9 @@
       <c r="I39" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="J39" s="430"/>
-      <c r="K39" s="395"/>
-      <c r="L39" s="395"/>
+      <c r="J39" s="416"/>
+      <c r="K39" s="400"/>
+      <c r="L39" s="400"/>
       <c r="M39" s="35"/>
     </row>
     <row r="40" spans="1:17" ht="14.4">
@@ -33707,9 +33707,9 @@
       <c r="I40" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="J40" s="395"/>
-      <c r="K40" s="395"/>
-      <c r="L40" s="395"/>
+      <c r="J40" s="400"/>
+      <c r="K40" s="400"/>
+      <c r="L40" s="400"/>
       <c r="M40" s="35"/>
     </row>
     <row r="41" spans="1:17" ht="14.4">
@@ -33738,9 +33738,9 @@
       <c r="I41" s="41" t="s">
         <v>224</v>
       </c>
-      <c r="J41" s="395"/>
-      <c r="K41" s="395"/>
-      <c r="L41" s="395"/>
+      <c r="J41" s="400"/>
+      <c r="K41" s="400"/>
+      <c r="L41" s="400"/>
       <c r="M41" s="35"/>
     </row>
     <row r="42" spans="1:17" ht="14.4">
@@ -33769,9 +33769,9 @@
       <c r="I42" s="185" t="s">
         <v>224</v>
       </c>
-      <c r="J42" s="430"/>
-      <c r="K42" s="395"/>
-      <c r="L42" s="395"/>
+      <c r="J42" s="416"/>
+      <c r="K42" s="400"/>
+      <c r="L42" s="400"/>
       <c r="M42" s="35"/>
     </row>
     <row r="43" spans="1:17" ht="14.4">
@@ -33800,9 +33800,9 @@
       <c r="I43" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="J43" s="395"/>
-      <c r="K43" s="395"/>
-      <c r="L43" s="395"/>
+      <c r="J43" s="400"/>
+      <c r="K43" s="400"/>
+      <c r="L43" s="400"/>
       <c r="M43" s="35"/>
     </row>
     <row r="44" spans="1:17" ht="14.4">
@@ -33831,9 +33831,9 @@
       <c r="I44" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="J44" s="395"/>
-      <c r="K44" s="395"/>
-      <c r="L44" s="395"/>
+      <c r="J44" s="400"/>
+      <c r="K44" s="400"/>
+      <c r="L44" s="400"/>
       <c r="M44" s="35"/>
     </row>
     <row r="45" spans="1:17" ht="14.4">
@@ -34026,103 +34026,103 @@
     </row>
     <row r="53" spans="1:17" ht="25.5" customHeight="1">
       <c r="A53" s="211"/>
-      <c r="B53" s="434" t="s">
+      <c r="B53" s="417" t="s">
         <v>363</v>
       </c>
-      <c r="C53" s="391"/>
-      <c r="D53" s="391"/>
-      <c r="E53" s="391"/>
-      <c r="F53" s="391"/>
-      <c r="G53" s="391"/>
-      <c r="H53" s="391"/>
-      <c r="I53" s="391"/>
-      <c r="J53" s="391"/>
-      <c r="K53" s="391"/>
-      <c r="L53" s="392"/>
+      <c r="C53" s="392"/>
+      <c r="D53" s="392"/>
+      <c r="E53" s="392"/>
+      <c r="F53" s="392"/>
+      <c r="G53" s="392"/>
+      <c r="H53" s="392"/>
+      <c r="I53" s="392"/>
+      <c r="J53" s="392"/>
+      <c r="K53" s="392"/>
+      <c r="L53" s="393"/>
       <c r="Q53" s="35"/>
     </row>
     <row r="54" spans="1:17" ht="20.25" customHeight="1">
       <c r="A54" s="34"/>
-      <c r="B54" s="426" t="s">
+      <c r="B54" s="418" t="s">
         <v>3</v>
       </c>
       <c r="C54" s="195" t="s">
         <v>329</v>
       </c>
       <c r="D54" s="195"/>
-      <c r="E54" s="414" t="s">
+      <c r="E54" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="F54" s="426" t="s">
+      <c r="F54" s="418" t="s">
         <v>5</v>
       </c>
       <c r="G54" s="238" t="s">
         <v>328</v>
       </c>
       <c r="H54" s="195"/>
-      <c r="I54" s="414" t="s">
+      <c r="I54" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="J54" s="426" t="s">
+      <c r="J54" s="418" t="s">
         <v>68</v>
       </c>
       <c r="K54" s="195" t="s">
         <v>220</v>
       </c>
       <c r="L54" s="239"/>
-      <c r="M54" s="414" t="s">
+      <c r="M54" s="411" t="s">
         <v>327</v>
       </c>
       <c r="Q54" s="35"/>
     </row>
     <row r="55" spans="1:17" ht="20.25" customHeight="1">
       <c r="A55" s="34"/>
-      <c r="B55" s="413"/>
+      <c r="B55" s="412"/>
       <c r="C55" s="195">
         <v>105</v>
       </c>
       <c r="D55" s="195"/>
-      <c r="E55" s="413"/>
-      <c r="F55" s="413"/>
+      <c r="E55" s="412"/>
+      <c r="F55" s="412"/>
       <c r="G55" s="240">
         <v>108</v>
       </c>
       <c r="H55" s="195"/>
-      <c r="I55" s="413"/>
-      <c r="J55" s="413"/>
+      <c r="I55" s="412"/>
+      <c r="J55" s="412"/>
       <c r="K55" s="195">
         <v>106</v>
       </c>
       <c r="L55" s="239"/>
-      <c r="M55" s="413"/>
+      <c r="M55" s="412"/>
       <c r="Q55" s="35"/>
     </row>
     <row r="56" spans="1:17" ht="23.25" customHeight="1">
       <c r="A56" s="34"/>
-      <c r="B56" s="408"/>
+      <c r="B56" s="402"/>
       <c r="C56" s="241" t="s">
         <v>7</v>
       </c>
       <c r="D56" s="241" t="s">
         <v>8</v>
       </c>
-      <c r="E56" s="408"/>
-      <c r="F56" s="408"/>
+      <c r="E56" s="402"/>
+      <c r="F56" s="402"/>
       <c r="G56" s="241" t="s">
         <v>7</v>
       </c>
       <c r="H56" s="241" t="s">
         <v>8</v>
       </c>
-      <c r="I56" s="408"/>
-      <c r="J56" s="408"/>
+      <c r="I56" s="402"/>
+      <c r="J56" s="402"/>
       <c r="K56" s="241" t="s">
         <v>7</v>
       </c>
       <c r="L56" s="241" t="s">
         <v>8</v>
       </c>
-      <c r="M56" s="408"/>
+      <c r="M56" s="402"/>
       <c r="Q56" s="35"/>
     </row>
     <row r="57" spans="1:17" ht="14.4">
@@ -34574,52 +34574,52 @@
     </row>
     <row r="72" spans="1:19" ht="24" customHeight="1">
       <c r="A72" s="211"/>
-      <c r="B72" s="435" t="s">
+      <c r="B72" s="413" t="s">
         <v>300</v>
       </c>
-      <c r="C72" s="391"/>
-      <c r="D72" s="391"/>
-      <c r="E72" s="391"/>
-      <c r="F72" s="391"/>
-      <c r="G72" s="391"/>
-      <c r="H72" s="391"/>
-      <c r="I72" s="391"/>
-      <c r="J72" s="391"/>
-      <c r="K72" s="391"/>
-      <c r="L72" s="392"/>
+      <c r="C72" s="392"/>
+      <c r="D72" s="392"/>
+      <c r="E72" s="392"/>
+      <c r="F72" s="392"/>
+      <c r="G72" s="392"/>
+      <c r="H72" s="392"/>
+      <c r="I72" s="392"/>
+      <c r="J72" s="392"/>
+      <c r="K72" s="392"/>
+      <c r="L72" s="393"/>
       <c r="M72" s="200"/>
       <c r="Q72" s="35"/>
     </row>
     <row r="73" spans="1:19" ht="21.75" customHeight="1">
       <c r="A73" s="34"/>
-      <c r="B73" s="427" t="s">
+      <c r="B73" s="424" t="s">
         <v>0</v>
       </c>
       <c r="C73" s="248" t="s">
         <v>328</v>
       </c>
       <c r="D73" s="248"/>
-      <c r="E73" s="414" t="s">
+      <c r="E73" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="F73" s="415" t="s">
+      <c r="F73" s="414" t="s">
         <v>5</v>
       </c>
       <c r="G73" s="206" t="s">
         <v>370</v>
       </c>
       <c r="H73" s="206"/>
-      <c r="I73" s="414" t="s">
+      <c r="I73" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="J73" s="415" t="s">
+      <c r="J73" s="414" t="s">
         <v>68</v>
       </c>
       <c r="K73" s="72" t="s">
         <v>329</v>
       </c>
       <c r="L73" s="72"/>
-      <c r="M73" s="414" t="s">
+      <c r="M73" s="411" t="s">
         <v>327</v>
       </c>
       <c r="N73" s="34"/>
@@ -34631,24 +34631,24 @@
     </row>
     <row r="74" spans="1:19" ht="21.75" customHeight="1">
       <c r="A74" s="34"/>
-      <c r="B74" s="413"/>
+      <c r="B74" s="412"/>
       <c r="C74" s="248">
         <v>108</v>
       </c>
       <c r="D74" s="248"/>
-      <c r="E74" s="413"/>
-      <c r="F74" s="413"/>
+      <c r="E74" s="412"/>
+      <c r="F74" s="412"/>
       <c r="G74" s="206">
         <v>106</v>
       </c>
       <c r="H74" s="206"/>
-      <c r="I74" s="413"/>
-      <c r="J74" s="413"/>
+      <c r="I74" s="412"/>
+      <c r="J74" s="412"/>
       <c r="K74" s="72">
         <v>105</v>
       </c>
       <c r="L74" s="72"/>
-      <c r="M74" s="413"/>
+      <c r="M74" s="412"/>
       <c r="N74" s="34"/>
       <c r="O74" s="34"/>
       <c r="P74" s="34"/>
@@ -34658,30 +34658,30 @@
     </row>
     <row r="75" spans="1:19" ht="27" customHeight="1">
       <c r="A75" s="34"/>
-      <c r="B75" s="408"/>
+      <c r="B75" s="402"/>
       <c r="C75" s="249" t="s">
         <v>7</v>
       </c>
       <c r="D75" s="249" t="s">
         <v>8</v>
       </c>
-      <c r="E75" s="408"/>
-      <c r="F75" s="408"/>
+      <c r="E75" s="402"/>
+      <c r="F75" s="402"/>
       <c r="G75" s="73" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="I75" s="408"/>
-      <c r="J75" s="408"/>
+      <c r="I75" s="402"/>
+      <c r="J75" s="402"/>
       <c r="K75" s="73" t="s">
         <v>7</v>
       </c>
       <c r="L75" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="M75" s="408"/>
+      <c r="M75" s="402"/>
       <c r="N75" s="34"/>
       <c r="O75" s="39"/>
       <c r="P75" s="39"/>
@@ -35249,86 +35249,86 @@
     </row>
     <row r="90" spans="1:19" ht="14.4">
       <c r="A90" s="34"/>
-      <c r="B90" s="415" t="s">
+      <c r="B90" s="414" t="s">
         <v>243</v>
       </c>
       <c r="C90" s="72" t="s">
         <v>220</v>
       </c>
       <c r="D90" s="72"/>
-      <c r="E90" s="414" t="s">
+      <c r="E90" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="F90" s="415" t="s">
+      <c r="F90" s="414" t="s">
         <v>48</v>
       </c>
       <c r="G90" s="72" t="s">
         <v>386</v>
       </c>
       <c r="H90" s="72"/>
-      <c r="I90" s="414" t="s">
+      <c r="I90" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="J90" s="416" t="s">
+      <c r="J90" s="431" t="s">
         <v>135</v>
       </c>
       <c r="K90" s="72" t="s">
         <v>387</v>
       </c>
       <c r="L90" s="72"/>
-      <c r="M90" s="417" t="s">
+      <c r="M90" s="432" t="s">
         <v>327</v>
       </c>
       <c r="Q90" s="35"/>
     </row>
     <row r="91" spans="1:19" ht="14.4">
       <c r="A91" s="34"/>
-      <c r="B91" s="413"/>
+      <c r="B91" s="412"/>
       <c r="C91" s="72">
         <v>104</v>
       </c>
       <c r="D91" s="72"/>
-      <c r="E91" s="413"/>
-      <c r="F91" s="413"/>
+      <c r="E91" s="412"/>
+      <c r="F91" s="412"/>
       <c r="G91" s="72">
         <v>107</v>
       </c>
       <c r="H91" s="72"/>
-      <c r="I91" s="413"/>
-      <c r="J91" s="413"/>
+      <c r="I91" s="412"/>
+      <c r="J91" s="412"/>
       <c r="K91" s="72">
         <v>103</v>
       </c>
       <c r="L91" s="72"/>
-      <c r="M91" s="413"/>
+      <c r="M91" s="412"/>
       <c r="Q91" s="35"/>
     </row>
     <row r="92" spans="1:19" ht="24" customHeight="1">
       <c r="A92" s="34"/>
-      <c r="B92" s="408"/>
+      <c r="B92" s="402"/>
       <c r="C92" s="73" t="s">
         <v>7</v>
       </c>
       <c r="D92" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="E92" s="408"/>
-      <c r="F92" s="408"/>
+      <c r="E92" s="402"/>
+      <c r="F92" s="402"/>
       <c r="G92" s="73" t="s">
         <v>7</v>
       </c>
       <c r="H92" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="I92" s="408"/>
-      <c r="J92" s="408"/>
+      <c r="I92" s="402"/>
+      <c r="J92" s="402"/>
       <c r="K92" s="73" t="s">
         <v>7</v>
       </c>
       <c r="L92" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="M92" s="408"/>
+      <c r="M92" s="402"/>
       <c r="Q92" s="35"/>
     </row>
     <row r="93" spans="1:19" ht="14.4">
@@ -35788,91 +35788,91 @@
     </row>
     <row r="107" spans="1:27" ht="21">
       <c r="A107" s="58"/>
-      <c r="B107" s="418" t="s">
+      <c r="B107" s="433" t="s">
         <v>302</v>
       </c>
-      <c r="C107" s="398"/>
-      <c r="D107" s="398"/>
-      <c r="E107" s="398"/>
-      <c r="F107" s="398"/>
-      <c r="G107" s="398"/>
-      <c r="H107" s="398"/>
-      <c r="I107" s="398"/>
-      <c r="J107" s="398"/>
-      <c r="K107" s="398"/>
-      <c r="L107" s="399"/>
+      <c r="C107" s="407"/>
+      <c r="D107" s="407"/>
+      <c r="E107" s="407"/>
+      <c r="F107" s="407"/>
+      <c r="G107" s="407"/>
+      <c r="H107" s="407"/>
+      <c r="I107" s="407"/>
+      <c r="J107" s="407"/>
+      <c r="K107" s="407"/>
+      <c r="L107" s="408"/>
       <c r="Q107" s="35"/>
     </row>
     <row r="108" spans="1:27" ht="14.4">
       <c r="A108" s="47"/>
-      <c r="B108" s="407" t="s">
+      <c r="B108" s="401" t="s">
         <v>3</v>
       </c>
       <c r="C108" s="168" t="s">
         <v>352</v>
       </c>
       <c r="D108" s="168"/>
-      <c r="E108" s="414" t="s">
+      <c r="E108" s="411" t="s">
         <v>327</v>
       </c>
-      <c r="F108" s="407"/>
+      <c r="F108" s="401"/>
       <c r="G108" s="168"/>
       <c r="H108" s="168"/>
-      <c r="I108" s="414" t="s">
+      <c r="I108" s="411" t="s">
         <v>398</v>
       </c>
-      <c r="J108" s="407"/>
+      <c r="J108" s="401"/>
       <c r="K108" s="168"/>
       <c r="L108" s="168"/>
-      <c r="M108" s="414" t="s">
+      <c r="M108" s="411" t="s">
         <v>327</v>
       </c>
       <c r="Q108" s="35"/>
     </row>
     <row r="109" spans="1:27" ht="14.4">
       <c r="A109" s="47"/>
-      <c r="B109" s="413"/>
+      <c r="B109" s="412"/>
       <c r="C109" s="168">
         <v>106</v>
       </c>
       <c r="D109" s="168"/>
-      <c r="E109" s="413"/>
-      <c r="F109" s="413"/>
+      <c r="E109" s="412"/>
+      <c r="F109" s="412"/>
       <c r="G109" s="168"/>
       <c r="H109" s="168"/>
-      <c r="I109" s="413"/>
-      <c r="J109" s="413"/>
+      <c r="I109" s="412"/>
+      <c r="J109" s="412"/>
       <c r="K109" s="168"/>
       <c r="L109" s="168"/>
-      <c r="M109" s="413"/>
+      <c r="M109" s="412"/>
       <c r="Q109" s="35"/>
     </row>
     <row r="110" spans="1:27" ht="22.5" customHeight="1">
       <c r="A110" s="47"/>
-      <c r="B110" s="408"/>
+      <c r="B110" s="402"/>
       <c r="C110" s="169" t="s">
         <v>7</v>
       </c>
       <c r="D110" s="169" t="s">
         <v>8</v>
       </c>
-      <c r="E110" s="408"/>
-      <c r="F110" s="408"/>
+      <c r="E110" s="402"/>
+      <c r="F110" s="402"/>
       <c r="G110" s="169" t="s">
         <v>7</v>
       </c>
       <c r="H110" s="169" t="s">
         <v>8</v>
       </c>
-      <c r="I110" s="408"/>
-      <c r="J110" s="408"/>
+      <c r="I110" s="402"/>
+      <c r="J110" s="402"/>
       <c r="K110" s="169" t="s">
         <v>7</v>
       </c>
       <c r="L110" s="169" t="s">
         <v>8</v>
       </c>
-      <c r="M110" s="408"/>
+      <c r="M110" s="402"/>
       <c r="Q110" s="35"/>
     </row>
     <row r="111" spans="1:27" ht="14.4">
@@ -35901,8 +35901,8 @@
       <c r="K111" s="98"/>
       <c r="L111" s="12"/>
       <c r="M111" s="45"/>
-      <c r="N111" s="424"/>
-      <c r="O111" s="395"/>
+      <c r="N111" s="421"/>
+      <c r="O111" s="400"/>
       <c r="Q111" s="35"/>
     </row>
     <row r="112" spans="1:27" ht="14.4">
@@ -35931,8 +35931,8 @@
       <c r="K112" s="26"/>
       <c r="L112" s="20"/>
       <c r="M112" s="45"/>
-      <c r="N112" s="395"/>
-      <c r="O112" s="395"/>
+      <c r="N112" s="400"/>
+      <c r="O112" s="400"/>
       <c r="Q112" s="35"/>
     </row>
     <row r="113" spans="1:17" ht="14.4">
@@ -35961,8 +35961,8 @@
       <c r="K113" s="15"/>
       <c r="L113" s="12"/>
       <c r="M113" s="45"/>
-      <c r="N113" s="395"/>
-      <c r="O113" s="395"/>
+      <c r="N113" s="400"/>
+      <c r="O113" s="400"/>
       <c r="Q113" s="35"/>
     </row>
     <row r="114" spans="1:17" ht="15.6">
@@ -35991,8 +35991,8 @@
       <c r="K114" s="15"/>
       <c r="L114" s="12"/>
       <c r="M114" s="45"/>
-      <c r="N114" s="395"/>
-      <c r="O114" s="395"/>
+      <c r="N114" s="400"/>
+      <c r="O114" s="400"/>
       <c r="Q114" s="35"/>
     </row>
     <row r="115" spans="1:17" ht="14.4">
@@ -36021,8 +36021,8 @@
       <c r="K115" s="17"/>
       <c r="L115" s="17"/>
       <c r="M115" s="185"/>
-      <c r="N115" s="395"/>
-      <c r="O115" s="395"/>
+      <c r="N115" s="400"/>
+      <c r="O115" s="400"/>
       <c r="Q115" s="35"/>
     </row>
     <row r="116" spans="1:17" ht="14.4">
@@ -38980,22 +38980,25 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="M73:M75"/>
-    <mergeCell ref="B72:L72"/>
-    <mergeCell ref="E73:E75"/>
-    <mergeCell ref="F73:F75"/>
-    <mergeCell ref="I73:I75"/>
-    <mergeCell ref="J73:J75"/>
-    <mergeCell ref="I54:I56"/>
-    <mergeCell ref="M54:M56"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="F36:F38"/>
-    <mergeCell ref="I36:I38"/>
-    <mergeCell ref="J39:L41"/>
-    <mergeCell ref="J42:L44"/>
-    <mergeCell ref="B53:L53"/>
-    <mergeCell ref="E54:E56"/>
-    <mergeCell ref="J54:J56"/>
+    <mergeCell ref="F108:F110"/>
+    <mergeCell ref="I108:I110"/>
+    <mergeCell ref="J108:J110"/>
+    <mergeCell ref="M108:M110"/>
+    <mergeCell ref="E90:E92"/>
+    <mergeCell ref="F90:F92"/>
+    <mergeCell ref="I90:I92"/>
+    <mergeCell ref="J90:J92"/>
+    <mergeCell ref="M90:M92"/>
+    <mergeCell ref="B107:L107"/>
+    <mergeCell ref="E108:E110"/>
+    <mergeCell ref="B1:N1"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="F3:F5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="M3:M5"/>
+    <mergeCell ref="B3:B5"/>
     <mergeCell ref="M19:M21"/>
     <mergeCell ref="O22:O25"/>
     <mergeCell ref="N111:O115"/>
@@ -39012,25 +39015,22 @@
     <mergeCell ref="K19:L20"/>
     <mergeCell ref="B35:L35"/>
     <mergeCell ref="F54:F56"/>
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="F3:F5"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="M3:M5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="F108:F110"/>
-    <mergeCell ref="I108:I110"/>
-    <mergeCell ref="J108:J110"/>
-    <mergeCell ref="M108:M110"/>
-    <mergeCell ref="E90:E92"/>
-    <mergeCell ref="F90:F92"/>
-    <mergeCell ref="I90:I92"/>
-    <mergeCell ref="J90:J92"/>
-    <mergeCell ref="M90:M92"/>
-    <mergeCell ref="B107:L107"/>
-    <mergeCell ref="E108:E110"/>
+    <mergeCell ref="I54:I56"/>
+    <mergeCell ref="M54:M56"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="F36:F38"/>
+    <mergeCell ref="I36:I38"/>
+    <mergeCell ref="J39:L41"/>
+    <mergeCell ref="J42:L44"/>
+    <mergeCell ref="B53:L53"/>
+    <mergeCell ref="E54:E56"/>
+    <mergeCell ref="J54:J56"/>
+    <mergeCell ref="M73:M75"/>
+    <mergeCell ref="B72:L72"/>
+    <mergeCell ref="E73:E75"/>
+    <mergeCell ref="F73:F75"/>
+    <mergeCell ref="I73:I75"/>
+    <mergeCell ref="J73:J75"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -39055,25 +39055,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="29.25" customHeight="1">
-      <c r="A1" s="436" t="s">
+      <c r="A1" s="434" t="s">
         <v>479</v>
       </c>
-      <c r="B1" s="395"/>
-      <c r="C1" s="395"/>
-      <c r="D1" s="395"/>
-      <c r="E1" s="395"/>
-      <c r="F1" s="395"/>
-      <c r="G1" s="395"/>
+      <c r="B1" s="400"/>
+      <c r="C1" s="400"/>
+      <c r="D1" s="400"/>
+      <c r="E1" s="400"/>
+      <c r="F1" s="400"/>
+      <c r="G1" s="400"/>
     </row>
     <row r="2" spans="1:8" ht="14.4">
-      <c r="A2" s="421" t="s">
+      <c r="A2" s="422" t="s">
         <v>480</v>
       </c>
       <c r="B2" s="179" t="s">
         <v>344</v>
       </c>
       <c r="C2" s="179"/>
-      <c r="E2" s="421" t="s">
+      <c r="E2" s="422" t="s">
         <v>481</v>
       </c>
       <c r="F2" s="179" t="s">
@@ -39082,14 +39082,14 @@
       <c r="G2" s="179"/>
     </row>
     <row r="3" spans="1:8" ht="14.4">
-      <c r="A3" s="413"/>
+      <c r="A3" s="412"/>
       <c r="B3" s="179">
         <v>108</v>
       </c>
       <c r="C3" s="179" t="s">
         <v>482</v>
       </c>
-      <c r="E3" s="413"/>
+      <c r="E3" s="412"/>
       <c r="F3" s="179">
         <v>107</v>
       </c>
@@ -39098,14 +39098,14 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="14.4">
-      <c r="A4" s="408"/>
+      <c r="A4" s="402"/>
       <c r="B4" s="179" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="179" t="s">
         <v>483</v>
       </c>
-      <c r="E4" s="408"/>
+      <c r="E4" s="402"/>
       <c r="F4" s="179" t="s">
         <v>7</v>
       </c>
@@ -39551,78 +39551,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27" customHeight="1">
-      <c r="A1" s="438" t="s">
+      <c r="A1" s="436" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="395"/>
-      <c r="C1" s="395"/>
-      <c r="D1" s="395"/>
-      <c r="E1" s="395"/>
-      <c r="F1" s="395"/>
-      <c r="G1" s="395"/>
-      <c r="H1" s="395"/>
-      <c r="I1" s="395"/>
-      <c r="J1" s="395"/>
-      <c r="K1" s="395"/>
+      <c r="B1" s="400"/>
+      <c r="C1" s="400"/>
+      <c r="D1" s="400"/>
+      <c r="E1" s="400"/>
+      <c r="F1" s="400"/>
+      <c r="G1" s="400"/>
+      <c r="H1" s="400"/>
+      <c r="I1" s="400"/>
+      <c r="J1" s="400"/>
+      <c r="K1" s="400"/>
       <c r="M1" s="270"/>
       <c r="N1" s="6" t="s">
         <v>505</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="25.8">
-      <c r="A2" s="439" t="s">
+      <c r="A2" s="437" t="s">
         <v>506</v>
       </c>
-      <c r="B2" s="410"/>
-      <c r="C2" s="410"/>
-      <c r="D2" s="410"/>
-      <c r="E2" s="410"/>
-      <c r="F2" s="410"/>
-      <c r="G2" s="410"/>
-      <c r="H2" s="410"/>
-      <c r="I2" s="410"/>
-      <c r="J2" s="410"/>
-      <c r="K2" s="411"/>
+      <c r="B2" s="404"/>
+      <c r="C2" s="404"/>
+      <c r="D2" s="404"/>
+      <c r="E2" s="404"/>
+      <c r="F2" s="404"/>
+      <c r="G2" s="404"/>
+      <c r="H2" s="404"/>
+      <c r="I2" s="404"/>
+      <c r="J2" s="404"/>
+      <c r="K2" s="405"/>
       <c r="L2" s="282"/>
       <c r="M2" s="282"/>
       <c r="N2" s="282"/>
       <c r="O2" s="282"/>
     </row>
     <row r="3" spans="1:15" ht="25.8">
-      <c r="A3" s="412"/>
-      <c r="B3" s="398"/>
-      <c r="C3" s="398"/>
-      <c r="D3" s="398"/>
-      <c r="E3" s="398"/>
-      <c r="F3" s="398"/>
-      <c r="G3" s="398"/>
-      <c r="H3" s="398"/>
-      <c r="I3" s="398"/>
-      <c r="J3" s="398"/>
-      <c r="K3" s="399"/>
+      <c r="A3" s="406"/>
+      <c r="B3" s="407"/>
+      <c r="C3" s="407"/>
+      <c r="D3" s="407"/>
+      <c r="E3" s="407"/>
+      <c r="F3" s="407"/>
+      <c r="G3" s="407"/>
+      <c r="H3" s="407"/>
+      <c r="I3" s="407"/>
+      <c r="J3" s="407"/>
+      <c r="K3" s="408"/>
       <c r="L3" s="282"/>
       <c r="M3" s="282"/>
       <c r="N3" s="282"/>
       <c r="O3" s="282"/>
     </row>
     <row r="5" spans="1:15" ht="18">
-      <c r="A5" s="440" t="s">
+      <c r="A5" s="438" t="s">
         <v>507</v>
       </c>
-      <c r="B5" s="391"/>
-      <c r="C5" s="392"/>
+      <c r="B5" s="392"/>
+      <c r="C5" s="393"/>
       <c r="D5" s="275"/>
-      <c r="E5" s="440" t="s">
+      <c r="E5" s="438" t="s">
         <v>508</v>
       </c>
-      <c r="F5" s="391"/>
-      <c r="G5" s="392"/>
+      <c r="F5" s="392"/>
+      <c r="G5" s="393"/>
       <c r="H5" s="283"/>
-      <c r="I5" s="440" t="s">
+      <c r="I5" s="438" t="s">
         <v>509</v>
       </c>
-      <c r="J5" s="391"/>
-      <c r="K5" s="392"/>
+      <c r="J5" s="392"/>
+      <c r="K5" s="393"/>
     </row>
     <row r="6" spans="1:15" ht="18">
       <c r="A6" s="284"/>
@@ -40070,7 +40070,9 @@
       <c r="K17" s="272">
         <v>2018</v>
       </c>
-      <c r="L17" s="62"/>
+      <c r="L17" s="185">
+        <v>5414582109</v>
+      </c>
     </row>
     <row r="18" spans="1:16" ht="19.8">
       <c r="A18" s="45">
@@ -40106,7 +40108,9 @@
       <c r="K18" s="295">
         <v>2018</v>
       </c>
-      <c r="L18" s="62"/>
+      <c r="L18" s="185">
+        <v>5422785361</v>
+      </c>
     </row>
     <row r="19" spans="1:16" ht="17.399999999999999">
       <c r="E19" s="45"/>
@@ -40116,42 +40120,42 @@
       <c r="L19" s="32"/>
     </row>
     <row r="20" spans="1:16" ht="14.4">
-      <c r="A20" s="441" t="s">
+      <c r="A20" s="439" t="s">
         <v>518</v>
       </c>
-      <c r="B20" s="410"/>
-      <c r="C20" s="410"/>
-      <c r="D20" s="410"/>
-      <c r="E20" s="410"/>
-      <c r="F20" s="410"/>
-      <c r="G20" s="410"/>
-      <c r="H20" s="410"/>
-      <c r="I20" s="410"/>
-      <c r="J20" s="410"/>
-      <c r="K20" s="410"/>
-      <c r="L20" s="410"/>
-      <c r="M20" s="410"/>
-      <c r="N20" s="410"/>
-      <c r="O20" s="410"/>
-      <c r="P20" s="411"/>
+      <c r="B20" s="404"/>
+      <c r="C20" s="404"/>
+      <c r="D20" s="404"/>
+      <c r="E20" s="404"/>
+      <c r="F20" s="404"/>
+      <c r="G20" s="404"/>
+      <c r="H20" s="404"/>
+      <c r="I20" s="404"/>
+      <c r="J20" s="404"/>
+      <c r="K20" s="404"/>
+      <c r="L20" s="404"/>
+      <c r="M20" s="404"/>
+      <c r="N20" s="404"/>
+      <c r="O20" s="404"/>
+      <c r="P20" s="405"/>
     </row>
     <row r="21" spans="1:16" ht="14.4">
-      <c r="A21" s="412"/>
-      <c r="B21" s="398"/>
-      <c r="C21" s="398"/>
-      <c r="D21" s="398"/>
-      <c r="E21" s="398"/>
-      <c r="F21" s="398"/>
-      <c r="G21" s="398"/>
-      <c r="H21" s="398"/>
-      <c r="I21" s="398"/>
-      <c r="J21" s="398"/>
-      <c r="K21" s="398"/>
-      <c r="L21" s="398"/>
-      <c r="M21" s="398"/>
-      <c r="N21" s="398"/>
-      <c r="O21" s="398"/>
-      <c r="P21" s="399"/>
+      <c r="A21" s="406"/>
+      <c r="B21" s="407"/>
+      <c r="C21" s="407"/>
+      <c r="D21" s="407"/>
+      <c r="E21" s="407"/>
+      <c r="F21" s="407"/>
+      <c r="G21" s="407"/>
+      <c r="H21" s="407"/>
+      <c r="I21" s="407"/>
+      <c r="J21" s="407"/>
+      <c r="K21" s="407"/>
+      <c r="L21" s="407"/>
+      <c r="M21" s="407"/>
+      <c r="N21" s="407"/>
+      <c r="O21" s="407"/>
+      <c r="P21" s="408"/>
     </row>
     <row r="22" spans="1:16" ht="14.4">
       <c r="M22" s="35"/>
@@ -40159,28 +40163,28 @@
       <c r="O22" s="35"/>
     </row>
     <row r="23" spans="1:16" ht="14.4">
-      <c r="A23" s="437" t="s">
+      <c r="A23" s="435" t="s">
         <v>519</v>
       </c>
-      <c r="B23" s="391"/>
-      <c r="C23" s="392"/>
+      <c r="B23" s="392"/>
+      <c r="C23" s="393"/>
       <c r="D23" s="283"/>
-      <c r="E23" s="437" t="s">
+      <c r="E23" s="435" t="s">
         <v>520</v>
       </c>
-      <c r="F23" s="391"/>
-      <c r="G23" s="392"/>
+      <c r="F23" s="392"/>
+      <c r="G23" s="393"/>
       <c r="H23" s="283"/>
-      <c r="I23" s="437" t="s">
+      <c r="I23" s="435" t="s">
         <v>509</v>
       </c>
-      <c r="J23" s="391"/>
-      <c r="K23" s="392"/>
-      <c r="M23" s="437" t="s">
+      <c r="J23" s="392"/>
+      <c r="K23" s="393"/>
+      <c r="M23" s="435" t="s">
         <v>521</v>
       </c>
-      <c r="N23" s="391"/>
-      <c r="O23" s="392"/>
+      <c r="N23" s="392"/>
+      <c r="O23" s="393"/>
       <c r="P23" s="283"/>
     </row>
     <row r="24" spans="1:16" ht="14.4">
@@ -40721,7 +40725,9 @@
       <c r="O34" s="272">
         <v>2017</v>
       </c>
-      <c r="P34" s="45"/>
+      <c r="P34" s="45">
+        <v>5312353268</v>
+      </c>
     </row>
     <row r="35" spans="1:16" ht="18">
       <c r="A35" s="45">
@@ -40769,7 +40775,9 @@
       <c r="O35" s="272">
         <v>2017</v>
       </c>
-      <c r="P35" s="45"/>
+      <c r="P35" s="45">
+        <v>5312353268</v>
+      </c>
     </row>
     <row r="36" spans="1:16" ht="18">
       <c r="A36" s="45">
@@ -40817,7 +40825,9 @@
       <c r="O36" s="269">
         <v>2019</v>
       </c>
-      <c r="P36" s="45"/>
+      <c r="P36" s="45">
+        <v>5307978853</v>
+      </c>
     </row>
     <row r="37" spans="1:16" ht="14.4">
       <c r="E37" s="6"/>
@@ -40895,7 +40905,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd"/>
+  <pageSetup paperSize="9" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -40913,34 +40923,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="33" customHeight="1">
-      <c r="A1" s="444" t="s">
+      <c r="A1" s="440" t="s">
         <v>532</v>
       </c>
-      <c r="B1" s="395"/>
-      <c r="C1" s="395"/>
-      <c r="D1" s="395"/>
-      <c r="E1" s="395"/>
-      <c r="F1" s="395"/>
-      <c r="G1" s="395"/>
-      <c r="H1" s="395"/>
-      <c r="I1" s="395"/>
-      <c r="J1" s="395"/>
+      <c r="B1" s="400"/>
+      <c r="C1" s="400"/>
+      <c r="D1" s="400"/>
+      <c r="E1" s="400"/>
+      <c r="F1" s="400"/>
+      <c r="G1" s="400"/>
+      <c r="H1" s="400"/>
+      <c r="I1" s="400"/>
+      <c r="J1" s="400"/>
       <c r="K1" s="211"/>
       <c r="L1" s="211"/>
       <c r="M1" s="211"/>
       <c r="N1" s="35"/>
     </row>
     <row r="2" spans="1:14" ht="33" customHeight="1">
-      <c r="A2" s="445" t="s">
+      <c r="A2" s="441" t="s">
         <v>533</v>
       </c>
-      <c r="B2" s="391"/>
-      <c r="C2" s="391"/>
-      <c r="D2" s="391"/>
-      <c r="E2" s="391"/>
-      <c r="F2" s="391"/>
-      <c r="G2" s="391"/>
-      <c r="H2" s="392"/>
+      <c r="B2" s="392"/>
+      <c r="C2" s="392"/>
+      <c r="D2" s="392"/>
+      <c r="E2" s="392"/>
+      <c r="F2" s="392"/>
+      <c r="G2" s="392"/>
+      <c r="H2" s="393"/>
       <c r="I2" s="211"/>
       <c r="J2" s="211"/>
       <c r="K2" s="211"/>
@@ -40949,62 +40959,62 @@
       <c r="N2" s="35"/>
     </row>
     <row r="3" spans="1:14" ht="15.6">
-      <c r="A3" s="421"/>
+      <c r="A3" s="422"/>
       <c r="B3" s="305" t="s">
         <v>534</v>
       </c>
       <c r="C3" s="179"/>
-      <c r="D3" s="414"/>
-      <c r="E3" s="446"/>
+      <c r="D3" s="411"/>
+      <c r="E3" s="442"/>
       <c r="F3" s="306" t="s">
         <v>535</v>
       </c>
       <c r="G3" s="137"/>
-      <c r="H3" s="414"/>
-      <c r="I3" s="430"/>
+      <c r="H3" s="411"/>
+      <c r="I3" s="416"/>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
-      <c r="L3" s="422"/>
+      <c r="L3" s="419"/>
       <c r="M3" s="35"/>
       <c r="N3" s="35"/>
     </row>
     <row r="4" spans="1:14" ht="14.4">
-      <c r="A4" s="413"/>
+      <c r="A4" s="412"/>
       <c r="B4" s="179"/>
       <c r="C4" s="179"/>
-      <c r="D4" s="413"/>
-      <c r="E4" s="413"/>
+      <c r="D4" s="412"/>
+      <c r="E4" s="412"/>
       <c r="F4" s="137"/>
       <c r="G4" s="137"/>
-      <c r="H4" s="413"/>
-      <c r="I4" s="395"/>
+      <c r="H4" s="412"/>
+      <c r="I4" s="400"/>
       <c r="J4" s="34"/>
       <c r="K4" s="34"/>
-      <c r="L4" s="395"/>
+      <c r="L4" s="400"/>
       <c r="M4" s="35"/>
       <c r="N4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="14.4">
-      <c r="A5" s="408"/>
+      <c r="A5" s="402"/>
       <c r="B5" s="180" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="180" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="408"/>
-      <c r="E5" s="408"/>
+      <c r="D5" s="402"/>
+      <c r="E5" s="402"/>
       <c r="F5" s="140" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="140" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="408"/>
-      <c r="I5" s="395"/>
+      <c r="H5" s="402"/>
+      <c r="I5" s="400"/>
       <c r="J5" s="39"/>
       <c r="K5" s="39"/>
-      <c r="L5" s="395"/>
+      <c r="L5" s="400"/>
       <c r="M5" s="35"/>
       <c r="N5" s="35"/>
     </row>
@@ -41295,67 +41305,67 @@
       </c>
     </row>
     <row r="20" spans="1:12" ht="26.25" customHeight="1">
-      <c r="A20" s="432" t="s">
+      <c r="A20" s="428" t="s">
         <v>551</v>
       </c>
-      <c r="B20" s="391"/>
-      <c r="C20" s="391"/>
-      <c r="D20" s="391"/>
-      <c r="E20" s="391"/>
-      <c r="F20" s="391"/>
-      <c r="G20" s="391"/>
-      <c r="H20" s="392"/>
+      <c r="B20" s="392"/>
+      <c r="C20" s="392"/>
+      <c r="D20" s="392"/>
+      <c r="E20" s="392"/>
+      <c r="F20" s="392"/>
+      <c r="G20" s="392"/>
+      <c r="H20" s="393"/>
       <c r="I20" s="211"/>
       <c r="J20" s="211"/>
       <c r="K20" s="211"/>
       <c r="L20" s="35"/>
     </row>
     <row r="21" spans="1:12" ht="14.4">
-      <c r="A21" s="442"/>
+      <c r="A21" s="443"/>
       <c r="B21" s="310" t="s">
         <v>552</v>
       </c>
       <c r="C21" s="310"/>
-      <c r="D21" s="414"/>
-      <c r="E21" s="443"/>
+      <c r="D21" s="411"/>
+      <c r="E21" s="444"/>
       <c r="F21" s="148"/>
       <c r="G21" s="148"/>
-      <c r="H21" s="414"/>
+      <c r="H21" s="411"/>
       <c r="I21" s="34"/>
       <c r="J21" s="34"/>
       <c r="K21" s="34"/>
       <c r="L21" s="35"/>
     </row>
     <row r="22" spans="1:12" ht="14.4">
-      <c r="A22" s="413"/>
+      <c r="A22" s="412"/>
       <c r="B22" s="310"/>
       <c r="C22" s="310"/>
-      <c r="D22" s="413"/>
-      <c r="E22" s="413"/>
+      <c r="D22" s="412"/>
+      <c r="E22" s="412"/>
       <c r="F22" s="148"/>
       <c r="G22" s="148"/>
-      <c r="H22" s="413"/>
+      <c r="H22" s="412"/>
       <c r="I22" s="34"/>
       <c r="J22" s="34"/>
       <c r="K22" s="34"/>
     </row>
     <row r="23" spans="1:12" ht="14.4">
-      <c r="A23" s="408"/>
+      <c r="A23" s="402"/>
       <c r="B23" s="311" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="311" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="408"/>
-      <c r="E23" s="408"/>
+      <c r="D23" s="402"/>
+      <c r="E23" s="402"/>
       <c r="F23" s="151" t="s">
         <v>7</v>
       </c>
       <c r="G23" s="151" t="s">
         <v>8</v>
       </c>
-      <c r="H23" s="408"/>
+      <c r="H23" s="402"/>
       <c r="I23" s="34"/>
       <c r="J23" s="39"/>
       <c r="K23" s="39"/>
@@ -41662,6 +41672,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="H21:H23"/>
     <mergeCell ref="L3:L5"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:H2"/>
@@ -41670,11 +41685,6 @@
     <mergeCell ref="E3:E5"/>
     <mergeCell ref="I3:I5"/>
     <mergeCell ref="H3:H5"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="H21:H23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -41716,33 +41726,33 @@
     </row>
     <row r="2" spans="1:16" ht="21">
       <c r="A2" s="2"/>
-      <c r="B2" s="447" t="s">
+      <c r="B2" s="454" t="s">
         <v>567</v>
       </c>
-      <c r="C2" s="391"/>
-      <c r="D2" s="391"/>
-      <c r="E2" s="391"/>
-      <c r="F2" s="391"/>
-      <c r="G2" s="391"/>
-      <c r="H2" s="391"/>
-      <c r="I2" s="391"/>
-      <c r="J2" s="391"/>
-      <c r="K2" s="391"/>
-      <c r="L2" s="392"/>
+      <c r="C2" s="392"/>
+      <c r="D2" s="392"/>
+      <c r="E2" s="392"/>
+      <c r="F2" s="392"/>
+      <c r="G2" s="392"/>
+      <c r="H2" s="392"/>
+      <c r="I2" s="392"/>
+      <c r="J2" s="392"/>
+      <c r="K2" s="392"/>
+      <c r="L2" s="393"/>
     </row>
     <row r="3" spans="1:16" ht="14.4">
       <c r="A3" s="2"/>
-      <c r="B3" s="448" t="s">
+      <c r="B3" s="452" t="s">
         <v>568</v>
       </c>
-      <c r="C3" s="395"/>
-      <c r="D3" s="395"/>
+      <c r="C3" s="400"/>
+      <c r="D3" s="400"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="449" t="s">
+      <c r="F3" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="G3" s="391"/>
-      <c r="H3" s="392"/>
+      <c r="G3" s="392"/>
+      <c r="H3" s="393"/>
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:16" ht="14.4">
@@ -42082,17 +42092,17 @@
     </row>
     <row r="19" spans="1:9" ht="14.4">
       <c r="A19" s="2"/>
-      <c r="B19" s="450" t="s">
+      <c r="B19" s="455" t="s">
         <v>568</v>
       </c>
-      <c r="C19" s="398"/>
-      <c r="D19" s="399"/>
+      <c r="C19" s="407"/>
+      <c r="D19" s="408"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="449" t="s">
+      <c r="F19" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="G19" s="391"/>
-      <c r="H19" s="392"/>
+      <c r="G19" s="392"/>
+      <c r="H19" s="393"/>
       <c r="I19" s="2"/>
     </row>
     <row r="20" spans="1:9" ht="14.4">
@@ -42402,30 +42412,30 @@
       <c r="B34" s="451" t="s">
         <v>599</v>
       </c>
-      <c r="C34" s="391"/>
-      <c r="D34" s="391"/>
-      <c r="E34" s="391"/>
-      <c r="F34" s="391"/>
-      <c r="G34" s="391"/>
-      <c r="H34" s="391"/>
-      <c r="I34" s="391"/>
-      <c r="J34" s="391"/>
-      <c r="K34" s="391"/>
-      <c r="L34" s="392"/>
+      <c r="C34" s="392"/>
+      <c r="D34" s="392"/>
+      <c r="E34" s="392"/>
+      <c r="F34" s="392"/>
+      <c r="G34" s="392"/>
+      <c r="H34" s="392"/>
+      <c r="I34" s="392"/>
+      <c r="J34" s="392"/>
+      <c r="K34" s="392"/>
+      <c r="L34" s="393"/>
     </row>
     <row r="35" spans="1:12" ht="15.75" customHeight="1">
       <c r="A35" s="2"/>
-      <c r="B35" s="449" t="s">
+      <c r="B35" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="C35" s="391"/>
-      <c r="D35" s="392"/>
+      <c r="C35" s="392"/>
+      <c r="D35" s="393"/>
       <c r="E35" s="2"/>
-      <c r="F35" s="448" t="s">
+      <c r="F35" s="452" t="s">
         <v>568</v>
       </c>
-      <c r="G35" s="395"/>
-      <c r="H35" s="395"/>
+      <c r="G35" s="400"/>
+      <c r="H35" s="400"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
@@ -42802,33 +42812,33 @@
     </row>
     <row r="52" spans="1:12" ht="20.25" customHeight="1">
       <c r="A52" s="2"/>
-      <c r="B52" s="452" t="s">
+      <c r="B52" s="453" t="s">
         <v>615</v>
       </c>
-      <c r="C52" s="391"/>
-      <c r="D52" s="391"/>
-      <c r="E52" s="391"/>
-      <c r="F52" s="391"/>
-      <c r="G52" s="391"/>
-      <c r="H52" s="391"/>
-      <c r="I52" s="391"/>
-      <c r="J52" s="391"/>
-      <c r="K52" s="391"/>
-      <c r="L52" s="392"/>
+      <c r="C52" s="392"/>
+      <c r="D52" s="392"/>
+      <c r="E52" s="392"/>
+      <c r="F52" s="392"/>
+      <c r="G52" s="392"/>
+      <c r="H52" s="392"/>
+      <c r="I52" s="392"/>
+      <c r="J52" s="392"/>
+      <c r="K52" s="392"/>
+      <c r="L52" s="393"/>
     </row>
     <row r="53" spans="1:12" ht="20.25" customHeight="1">
       <c r="A53" s="2"/>
-      <c r="B53" s="449" t="s">
+      <c r="B53" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="C53" s="391"/>
-      <c r="D53" s="392"/>
+      <c r="C53" s="392"/>
+      <c r="D53" s="393"/>
       <c r="E53" s="2"/>
-      <c r="F53" s="449" t="s">
+      <c r="F53" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="G53" s="391"/>
-      <c r="H53" s="392"/>
+      <c r="G53" s="392"/>
+      <c r="H53" s="393"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
@@ -43248,23 +43258,23 @@
     </row>
     <row r="69" spans="1:12" ht="15.75" customHeight="1">
       <c r="A69" s="2"/>
-      <c r="B69" s="449" t="s">
+      <c r="B69" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="C69" s="391"/>
-      <c r="D69" s="392"/>
+      <c r="C69" s="392"/>
+      <c r="D69" s="393"/>
       <c r="E69" s="2"/>
-      <c r="F69" s="449" t="s">
+      <c r="F69" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="G69" s="391"/>
-      <c r="H69" s="392"/>
+      <c r="G69" s="392"/>
+      <c r="H69" s="393"/>
       <c r="I69" s="2"/>
-      <c r="J69" s="449" t="s">
+      <c r="J69" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="K69" s="391"/>
-      <c r="L69" s="392"/>
+      <c r="K69" s="392"/>
+      <c r="L69" s="393"/>
     </row>
     <row r="70" spans="1:12" ht="15.75" customHeight="1">
       <c r="A70" s="2"/>
@@ -43654,39 +43664,39 @@
     </row>
     <row r="85" spans="1:12" ht="15.75" customHeight="1">
       <c r="A85" s="2"/>
-      <c r="B85" s="453" t="s">
+      <c r="B85" s="450" t="s">
         <v>645</v>
       </c>
-      <c r="C85" s="391"/>
-      <c r="D85" s="391"/>
-      <c r="E85" s="391"/>
-      <c r="F85" s="391"/>
-      <c r="G85" s="391"/>
-      <c r="H85" s="391"/>
-      <c r="I85" s="391"/>
-      <c r="J85" s="391"/>
-      <c r="K85" s="391"/>
-      <c r="L85" s="392"/>
+      <c r="C85" s="392"/>
+      <c r="D85" s="392"/>
+      <c r="E85" s="392"/>
+      <c r="F85" s="392"/>
+      <c r="G85" s="392"/>
+      <c r="H85" s="392"/>
+      <c r="I85" s="392"/>
+      <c r="J85" s="392"/>
+      <c r="K85" s="392"/>
+      <c r="L85" s="393"/>
     </row>
     <row r="86" spans="1:12" ht="15.75" customHeight="1">
       <c r="A86" s="2"/>
-      <c r="B86" s="449" t="s">
+      <c r="B86" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="C86" s="391"/>
-      <c r="D86" s="392"/>
+      <c r="C86" s="392"/>
+      <c r="D86" s="393"/>
       <c r="E86" s="2"/>
-      <c r="F86" s="449" t="s">
+      <c r="F86" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="G86" s="391"/>
-      <c r="H86" s="392"/>
+      <c r="G86" s="392"/>
+      <c r="H86" s="393"/>
       <c r="I86" s="2"/>
-      <c r="J86" s="449" t="s">
+      <c r="J86" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="K86" s="391"/>
-      <c r="L86" s="392"/>
+      <c r="K86" s="392"/>
+      <c r="L86" s="393"/>
     </row>
     <row r="87" spans="1:12" ht="15.75" customHeight="1">
       <c r="A87" s="2"/>
@@ -44171,23 +44181,23 @@
     </row>
     <row r="103" spans="1:13" ht="15.75" customHeight="1">
       <c r="A103" s="2"/>
-      <c r="B103" s="449" t="s">
+      <c r="B103" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="C103" s="391"/>
-      <c r="D103" s="392"/>
+      <c r="C103" s="392"/>
+      <c r="D103" s="393"/>
       <c r="E103" s="2"/>
-      <c r="F103" s="449" t="s">
+      <c r="F103" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="G103" s="391"/>
-      <c r="H103" s="392"/>
+      <c r="G103" s="392"/>
+      <c r="H103" s="393"/>
       <c r="I103" s="2"/>
-      <c r="J103" s="449" t="s">
+      <c r="J103" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="K103" s="391"/>
-      <c r="L103" s="392"/>
+      <c r="K103" s="392"/>
+      <c r="L103" s="393"/>
     </row>
     <row r="104" spans="1:13" ht="15.75" customHeight="1">
       <c r="A104" s="2"/>
@@ -44634,11 +44644,11 @@
     </row>
     <row r="119" spans="1:12" ht="15.75" customHeight="1">
       <c r="A119" s="2"/>
-      <c r="B119" s="449" t="s">
+      <c r="B119" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="C119" s="391"/>
-      <c r="D119" s="392"/>
+      <c r="C119" s="392"/>
+      <c r="D119" s="393"/>
       <c r="E119" s="2"/>
       <c r="F119" s="2"/>
       <c r="G119" s="2"/>
@@ -44928,39 +44938,39 @@
     </row>
     <row r="135" spans="1:13" ht="15.75" customHeight="1">
       <c r="A135" s="2"/>
-      <c r="B135" s="397" t="s">
+      <c r="B135" s="447" t="s">
         <v>697</v>
       </c>
-      <c r="C135" s="391"/>
-      <c r="D135" s="391"/>
-      <c r="E135" s="391"/>
-      <c r="F135" s="391"/>
-      <c r="G135" s="391"/>
-      <c r="H135" s="391"/>
-      <c r="I135" s="391"/>
-      <c r="J135" s="391"/>
-      <c r="K135" s="391"/>
-      <c r="L135" s="392"/>
+      <c r="C135" s="392"/>
+      <c r="D135" s="392"/>
+      <c r="E135" s="392"/>
+      <c r="F135" s="392"/>
+      <c r="G135" s="392"/>
+      <c r="H135" s="392"/>
+      <c r="I135" s="392"/>
+      <c r="J135" s="392"/>
+      <c r="K135" s="392"/>
+      <c r="L135" s="393"/>
     </row>
     <row r="136" spans="1:13" ht="15.75" customHeight="1">
       <c r="A136" s="2"/>
-      <c r="B136" s="449" t="s">
+      <c r="B136" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="C136" s="391"/>
-      <c r="D136" s="392"/>
+      <c r="C136" s="392"/>
+      <c r="D136" s="393"/>
       <c r="E136" s="2"/>
-      <c r="F136" s="449" t="s">
+      <c r="F136" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="G136" s="391"/>
-      <c r="H136" s="392"/>
+      <c r="G136" s="392"/>
+      <c r="H136" s="393"/>
       <c r="I136" s="2"/>
-      <c r="J136" s="449" t="s">
+      <c r="J136" s="445" t="s">
         <v>568</v>
       </c>
-      <c r="K136" s="391"/>
-      <c r="L136" s="392"/>
+      <c r="K136" s="392"/>
+      <c r="L136" s="393"/>
     </row>
     <row r="137" spans="1:13" ht="15.75" customHeight="1">
       <c r="A137" s="2"/>
@@ -45453,14 +45463,14 @@
     </row>
     <row r="155" spans="1:12" ht="15.75" customHeight="1">
       <c r="A155" s="2"/>
-      <c r="B155" s="455" t="s">
+      <c r="B155" s="448" t="s">
         <v>722</v>
       </c>
-      <c r="C155" s="391"/>
-      <c r="D155" s="391"/>
-      <c r="E155" s="391"/>
-      <c r="F155" s="391"/>
-      <c r="G155" s="392"/>
+      <c r="C155" s="392"/>
+      <c r="D155" s="392"/>
+      <c r="E155" s="392"/>
+      <c r="F155" s="392"/>
+      <c r="G155" s="393"/>
       <c r="H155" s="2"/>
       <c r="I155" s="2"/>
       <c r="J155" s="2"/>
@@ -45490,10 +45500,10 @@
       <c r="D157" s="346" t="s">
         <v>8</v>
       </c>
-      <c r="E157" s="456" t="s">
+      <c r="E157" s="449" t="s">
         <v>723</v>
       </c>
-      <c r="F157" s="392"/>
+      <c r="F157" s="393"/>
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
       <c r="I157" s="2"/>
@@ -45534,10 +45544,10 @@
       <c r="D159" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="E159" s="454" t="s">
+      <c r="E159" s="446" t="s">
         <v>727</v>
       </c>
-      <c r="F159" s="392"/>
+      <c r="F159" s="393"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
       <c r="I159" s="2"/>
@@ -45640,8 +45650,8 @@
       </c>
       <c r="C164" s="334"/>
       <c r="D164" s="71"/>
-      <c r="E164" s="454"/>
-      <c r="F164" s="392"/>
+      <c r="E164" s="446"/>
+      <c r="F164" s="393"/>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
       <c r="I164" s="2"/>
@@ -57439,6 +57449,24 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="B34:L34"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="B52:L52"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="F53:H53"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="F69:H69"/>
+    <mergeCell ref="J69:L69"/>
+    <mergeCell ref="B85:L85"/>
+    <mergeCell ref="B86:D86"/>
+    <mergeCell ref="F86:H86"/>
+    <mergeCell ref="J86:L86"/>
     <mergeCell ref="B103:D103"/>
     <mergeCell ref="F103:H103"/>
     <mergeCell ref="J103:L103"/>
@@ -57451,24 +57479,6 @@
     <mergeCell ref="J136:L136"/>
     <mergeCell ref="B155:G155"/>
     <mergeCell ref="E157:F157"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="F69:H69"/>
-    <mergeCell ref="J69:L69"/>
-    <mergeCell ref="B85:L85"/>
-    <mergeCell ref="B86:D86"/>
-    <mergeCell ref="F86:H86"/>
-    <mergeCell ref="J86:L86"/>
-    <mergeCell ref="B34:L34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="B52:L52"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="F19:H19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -57509,19 +57519,19 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="21">
-      <c r="B2" s="447" t="s">
+      <c r="B2" s="454" t="s">
         <v>736</v>
       </c>
-      <c r="C2" s="391"/>
-      <c r="D2" s="391"/>
-      <c r="E2" s="391"/>
-      <c r="F2" s="391"/>
-      <c r="G2" s="391"/>
-      <c r="H2" s="391"/>
-      <c r="I2" s="391"/>
-      <c r="J2" s="391"/>
-      <c r="K2" s="391"/>
-      <c r="L2" s="392"/>
+      <c r="C2" s="392"/>
+      <c r="D2" s="392"/>
+      <c r="E2" s="392"/>
+      <c r="F2" s="392"/>
+      <c r="G2" s="392"/>
+      <c r="H2" s="392"/>
+      <c r="I2" s="392"/>
+      <c r="J2" s="392"/>
+      <c r="K2" s="392"/>
+      <c r="L2" s="393"/>
     </row>
     <row r="4" spans="1:12" ht="14.4">
       <c r="B4" s="313" t="s">
@@ -58173,16 +58183,16 @@
       <c r="B36" s="451" t="s">
         <v>599</v>
       </c>
-      <c r="C36" s="391"/>
-      <c r="D36" s="391"/>
-      <c r="E36" s="391"/>
-      <c r="F36" s="391"/>
-      <c r="G36" s="391"/>
-      <c r="H36" s="391"/>
-      <c r="I36" s="391"/>
-      <c r="J36" s="391"/>
-      <c r="K36" s="391"/>
-      <c r="L36" s="392"/>
+      <c r="C36" s="392"/>
+      <c r="D36" s="392"/>
+      <c r="E36" s="392"/>
+      <c r="F36" s="392"/>
+      <c r="G36" s="392"/>
+      <c r="H36" s="392"/>
+      <c r="I36" s="392"/>
+      <c r="J36" s="392"/>
+      <c r="K36" s="392"/>
+      <c r="L36" s="393"/>
     </row>
     <row r="37" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="38" spans="2:12" ht="15.75" customHeight="1">
@@ -58429,19 +58439,19 @@
       <c r="L53" s="2"/>
     </row>
     <row r="54" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B54" s="452" t="s">
+      <c r="B54" s="453" t="s">
         <v>615</v>
       </c>
-      <c r="C54" s="391"/>
-      <c r="D54" s="391"/>
-      <c r="E54" s="391"/>
-      <c r="F54" s="391"/>
-      <c r="G54" s="391"/>
-      <c r="H54" s="391"/>
-      <c r="I54" s="391"/>
-      <c r="J54" s="391"/>
-      <c r="K54" s="391"/>
-      <c r="L54" s="392"/>
+      <c r="C54" s="392"/>
+      <c r="D54" s="392"/>
+      <c r="E54" s="392"/>
+      <c r="F54" s="392"/>
+      <c r="G54" s="392"/>
+      <c r="H54" s="392"/>
+      <c r="I54" s="392"/>
+      <c r="J54" s="392"/>
+      <c r="K54" s="392"/>
+      <c r="L54" s="393"/>
     </row>
     <row r="55" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="56" spans="2:12" ht="15.75" customHeight="1">
@@ -59184,19 +59194,19 @@
     </row>
     <row r="86" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="87" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B87" s="453" t="s">
+      <c r="B87" s="450" t="s">
         <v>760</v>
       </c>
-      <c r="C87" s="391"/>
-      <c r="D87" s="391"/>
-      <c r="E87" s="391"/>
-      <c r="F87" s="391"/>
-      <c r="G87" s="391"/>
-      <c r="H87" s="391"/>
-      <c r="I87" s="391"/>
-      <c r="J87" s="391"/>
-      <c r="K87" s="391"/>
-      <c r="L87" s="392"/>
+      <c r="C87" s="392"/>
+      <c r="D87" s="392"/>
+      <c r="E87" s="392"/>
+      <c r="F87" s="392"/>
+      <c r="G87" s="392"/>
+      <c r="H87" s="392"/>
+      <c r="I87" s="392"/>
+      <c r="J87" s="392"/>
+      <c r="K87" s="392"/>
+      <c r="L87" s="393"/>
     </row>
     <row r="88" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="89" spans="2:12" ht="15.75" customHeight="1">
@@ -59992,19 +60002,19 @@
     <row r="119" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="120" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="121" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B121" s="397" t="s">
+      <c r="B121" s="447" t="s">
         <v>766</v>
       </c>
-      <c r="C121" s="391"/>
-      <c r="D121" s="391"/>
-      <c r="E121" s="391"/>
-      <c r="F121" s="391"/>
-      <c r="G121" s="391"/>
-      <c r="H121" s="391"/>
-      <c r="I121" s="391"/>
-      <c r="J121" s="391"/>
-      <c r="K121" s="391"/>
-      <c r="L121" s="392"/>
+      <c r="C121" s="392"/>
+      <c r="D121" s="392"/>
+      <c r="E121" s="392"/>
+      <c r="F121" s="392"/>
+      <c r="G121" s="392"/>
+      <c r="H121" s="392"/>
+      <c r="I121" s="392"/>
+      <c r="J121" s="392"/>
+      <c r="K121" s="392"/>
+      <c r="L121" s="393"/>
     </row>
     <row r="122" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="123" spans="2:12" ht="15.75" customHeight="1">
@@ -60417,14 +60427,14 @@
     <row r="139" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="140" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="141" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B141" s="455" t="s">
+      <c r="B141" s="448" t="s">
         <v>722</v>
       </c>
-      <c r="C141" s="391"/>
-      <c r="D141" s="391"/>
-      <c r="E141" s="391"/>
-      <c r="F141" s="391"/>
-      <c r="G141" s="392"/>
+      <c r="C141" s="392"/>
+      <c r="D141" s="392"/>
+      <c r="E141" s="392"/>
+      <c r="F141" s="392"/>
+      <c r="G141" s="393"/>
     </row>
     <row r="142" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="143" spans="2:12" ht="15.75" customHeight="1">
@@ -60435,10 +60445,10 @@
       <c r="D143" s="346" t="s">
         <v>8</v>
       </c>
-      <c r="E143" s="456" t="s">
+      <c r="E143" s="449" t="s">
         <v>723</v>
       </c>
-      <c r="F143" s="392"/>
+      <c r="F143" s="393"/>
     </row>
     <row r="144" spans="2:12" ht="15.75" customHeight="1">
       <c r="B144" s="7">
@@ -60467,10 +60477,10 @@
       <c r="D145" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="E145" s="454" t="s">
+      <c r="E145" s="446" t="s">
         <v>727</v>
       </c>
-      <c r="F145" s="392"/>
+      <c r="F145" s="393"/>
       <c r="K145" s="2"/>
     </row>
     <row r="146" spans="2:12" ht="15.75" customHeight="1">
@@ -60573,8 +60583,8 @@
       <c r="D151" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="E151" s="454"/>
-      <c r="F151" s="392"/>
+      <c r="E151" s="446"/>
+      <c r="F151" s="393"/>
     </row>
     <row r="152" spans="2:12" ht="15.75" customHeight="1">
       <c r="B152" s="7">
@@ -60582,8 +60592,8 @@
       </c>
       <c r="C152" s="7"/>
       <c r="D152" s="71"/>
-      <c r="E152" s="454"/>
-      <c r="F152" s="392"/>
+      <c r="E152" s="446"/>
+      <c r="F152" s="393"/>
       <c r="G152" s="2"/>
     </row>
     <row r="153" spans="2:12" ht="15.75" customHeight="1">
@@ -60592,8 +60602,8 @@
       </c>
       <c r="C153" s="71"/>
       <c r="D153" s="71"/>
-      <c r="E153" s="454"/>
-      <c r="F153" s="392"/>
+      <c r="E153" s="446"/>
+      <c r="F153" s="393"/>
     </row>
     <row r="154" spans="2:12" ht="15.75" customHeight="1">
       <c r="B154" s="7">
@@ -60601,8 +60611,8 @@
       </c>
       <c r="C154" s="334"/>
       <c r="D154" s="71"/>
-      <c r="E154" s="457"/>
-      <c r="F154" s="392"/>
+      <c r="E154" s="456"/>
+      <c r="F154" s="393"/>
     </row>
     <row r="155" spans="2:12" ht="15.75" customHeight="1">
       <c r="B155" s="7">
@@ -60610,8 +60620,8 @@
       </c>
       <c r="C155" s="334"/>
       <c r="D155" s="71"/>
-      <c r="E155" s="454"/>
-      <c r="F155" s="392"/>
+      <c r="E155" s="446"/>
+      <c r="F155" s="393"/>
     </row>
     <row r="156" spans="2:12" ht="15.75" customHeight="1">
       <c r="B156" s="7">
@@ -60619,8 +60629,8 @@
       </c>
       <c r="C156" s="334"/>
       <c r="D156" s="71"/>
-      <c r="E156" s="454"/>
-      <c r="F156" s="392"/>
+      <c r="E156" s="446"/>
+      <c r="F156" s="393"/>
     </row>
     <row r="157" spans="2:12" ht="15.75" customHeight="1">
       <c r="B157" s="7">
@@ -60628,8 +60638,8 @@
       </c>
       <c r="C157" s="7"/>
       <c r="D157" s="333"/>
-      <c r="E157" s="454"/>
-      <c r="F157" s="392"/>
+      <c r="E157" s="446"/>
+      <c r="F157" s="393"/>
     </row>
     <row r="158" spans="2:12" ht="15.75" customHeight="1">
       <c r="B158" s="7">
@@ -60637,8 +60647,8 @@
       </c>
       <c r="C158" s="334"/>
       <c r="D158" s="71"/>
-      <c r="E158" s="454"/>
-      <c r="F158" s="392"/>
+      <c r="E158" s="446"/>
+      <c r="F158" s="393"/>
     </row>
     <row r="159" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="160" spans="2:12" ht="15.75" customHeight="1"/>
@@ -61446,6 +61456,11 @@
     <row r="962" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B54:L54"/>
+    <mergeCell ref="B87:L87"/>
+    <mergeCell ref="B121:L121"/>
     <mergeCell ref="B141:G141"/>
     <mergeCell ref="E143:F143"/>
     <mergeCell ref="E157:F157"/>
@@ -61457,11 +61472,6 @@
     <mergeCell ref="E154:F154"/>
     <mergeCell ref="E155:F155"/>
     <mergeCell ref="E156:F156"/>
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="B54:L54"/>
-    <mergeCell ref="B87:L87"/>
-    <mergeCell ref="B121:L121"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape"/>
@@ -61502,19 +61512,19 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:11" ht="21">
-      <c r="A2" s="447" t="s">
+      <c r="A2" s="454" t="s">
         <v>736</v>
       </c>
-      <c r="B2" s="391"/>
-      <c r="C2" s="391"/>
-      <c r="D2" s="391"/>
-      <c r="E2" s="391"/>
-      <c r="F2" s="391"/>
-      <c r="G2" s="391"/>
-      <c r="H2" s="391"/>
-      <c r="I2" s="391"/>
-      <c r="J2" s="391"/>
-      <c r="K2" s="392"/>
+      <c r="B2" s="392"/>
+      <c r="C2" s="392"/>
+      <c r="D2" s="392"/>
+      <c r="E2" s="392"/>
+      <c r="F2" s="392"/>
+      <c r="G2" s="392"/>
+      <c r="H2" s="392"/>
+      <c r="I2" s="392"/>
+      <c r="J2" s="392"/>
+      <c r="K2" s="393"/>
     </row>
     <row r="3" spans="1:11" ht="14.4">
       <c r="A3" s="2"/>
@@ -62337,16 +62347,16 @@
       <c r="A36" s="451" t="s">
         <v>599</v>
       </c>
-      <c r="B36" s="391"/>
-      <c r="C36" s="391"/>
-      <c r="D36" s="391"/>
-      <c r="E36" s="391"/>
-      <c r="F36" s="391"/>
-      <c r="G36" s="391"/>
-      <c r="H36" s="391"/>
-      <c r="I36" s="391"/>
-      <c r="J36" s="391"/>
-      <c r="K36" s="392"/>
+      <c r="B36" s="392"/>
+      <c r="C36" s="392"/>
+      <c r="D36" s="392"/>
+      <c r="E36" s="392"/>
+      <c r="F36" s="392"/>
+      <c r="G36" s="392"/>
+      <c r="H36" s="392"/>
+      <c r="I36" s="392"/>
+      <c r="J36" s="392"/>
+      <c r="K36" s="393"/>
     </row>
     <row r="37" spans="1:11" ht="15.75" customHeight="1">
       <c r="A37" s="2"/>
@@ -62646,19 +62656,19 @@
       <c r="K53" s="2"/>
     </row>
     <row r="54" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A54" s="452" t="s">
+      <c r="A54" s="453" t="s">
         <v>615</v>
       </c>
-      <c r="B54" s="391"/>
-      <c r="C54" s="391"/>
-      <c r="D54" s="391"/>
-      <c r="E54" s="391"/>
-      <c r="F54" s="391"/>
-      <c r="G54" s="391"/>
-      <c r="H54" s="391"/>
-      <c r="I54" s="391"/>
-      <c r="J54" s="391"/>
-      <c r="K54" s="392"/>
+      <c r="B54" s="392"/>
+      <c r="C54" s="392"/>
+      <c r="D54" s="392"/>
+      <c r="E54" s="392"/>
+      <c r="F54" s="392"/>
+      <c r="G54" s="392"/>
+      <c r="H54" s="392"/>
+      <c r="I54" s="392"/>
+      <c r="J54" s="392"/>
+      <c r="K54" s="393"/>
     </row>
     <row r="55" spans="1:11" ht="15.75" customHeight="1">
       <c r="A55" s="2"/>
@@ -63509,19 +63519,19 @@
       <c r="K86" s="2"/>
     </row>
     <row r="87" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A87" s="453" t="s">
+      <c r="A87" s="450" t="s">
         <v>760</v>
       </c>
-      <c r="B87" s="391"/>
-      <c r="C87" s="391"/>
-      <c r="D87" s="391"/>
-      <c r="E87" s="391"/>
-      <c r="F87" s="391"/>
-      <c r="G87" s="391"/>
-      <c r="H87" s="391"/>
-      <c r="I87" s="391"/>
-      <c r="J87" s="391"/>
-      <c r="K87" s="392"/>
+      <c r="B87" s="392"/>
+      <c r="C87" s="392"/>
+      <c r="D87" s="392"/>
+      <c r="E87" s="392"/>
+      <c r="F87" s="392"/>
+      <c r="G87" s="392"/>
+      <c r="H87" s="392"/>
+      <c r="I87" s="392"/>
+      <c r="J87" s="392"/>
+      <c r="K87" s="393"/>
     </row>
     <row r="88" spans="1:11" ht="15.75" customHeight="1">
       <c r="A88" s="2"/>
@@ -64435,19 +64445,19 @@
       <c r="K120" s="2"/>
     </row>
     <row r="121" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A121" s="397" t="s">
+      <c r="A121" s="447" t="s">
         <v>766</v>
       </c>
-      <c r="B121" s="391"/>
-      <c r="C121" s="391"/>
-      <c r="D121" s="391"/>
-      <c r="E121" s="391"/>
-      <c r="F121" s="391"/>
-      <c r="G121" s="391"/>
-      <c r="H121" s="391"/>
-      <c r="I121" s="391"/>
-      <c r="J121" s="391"/>
-      <c r="K121" s="392"/>
+      <c r="B121" s="392"/>
+      <c r="C121" s="392"/>
+      <c r="D121" s="392"/>
+      <c r="E121" s="392"/>
+      <c r="F121" s="392"/>
+      <c r="G121" s="392"/>
+      <c r="H121" s="392"/>
+      <c r="I121" s="392"/>
+      <c r="J121" s="392"/>
+      <c r="K121" s="393"/>
     </row>
     <row r="122" spans="1:11" ht="15.75" customHeight="1">
       <c r="A122" s="2"/>
@@ -64943,14 +64953,14 @@
       <c r="K140" s="2"/>
     </row>
     <row r="141" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A141" s="455" t="s">
+      <c r="A141" s="448" t="s">
         <v>722</v>
       </c>
-      <c r="B141" s="391"/>
-      <c r="C141" s="391"/>
-      <c r="D141" s="391"/>
-      <c r="E141" s="391"/>
-      <c r="F141" s="392"/>
+      <c r="B141" s="392"/>
+      <c r="C141" s="392"/>
+      <c r="D141" s="392"/>
+      <c r="E141" s="392"/>
+      <c r="F141" s="393"/>
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
       <c r="I141" s="2"/>
@@ -64978,10 +64988,10 @@
       <c r="C143" s="346" t="s">
         <v>8</v>
       </c>
-      <c r="D143" s="456" t="s">
+      <c r="D143" s="449" t="s">
         <v>723</v>
       </c>
-      <c r="E143" s="392"/>
+      <c r="E143" s="393"/>
       <c r="F143" s="2"/>
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
@@ -65020,10 +65030,10 @@
       <c r="C145" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="D145" s="454" t="s">
+      <c r="D145" s="446" t="s">
         <v>727</v>
       </c>
-      <c r="E145" s="392"/>
+      <c r="E145" s="393"/>
       <c r="F145" s="2"/>
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
@@ -65144,8 +65154,8 @@
       <c r="C151" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="D151" s="454"/>
-      <c r="E151" s="392"/>
+      <c r="D151" s="446"/>
+      <c r="E151" s="393"/>
       <c r="F151" s="2"/>
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
@@ -65159,8 +65169,8 @@
       </c>
       <c r="B152" s="7"/>
       <c r="C152" s="71"/>
-      <c r="D152" s="454"/>
-      <c r="E152" s="392"/>
+      <c r="D152" s="446"/>
+      <c r="E152" s="393"/>
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
@@ -65174,8 +65184,8 @@
       </c>
       <c r="B153" s="71"/>
       <c r="C153" s="71"/>
-      <c r="D153" s="454"/>
-      <c r="E153" s="392"/>
+      <c r="D153" s="446"/>
+      <c r="E153" s="393"/>
       <c r="F153" s="2"/>
       <c r="G153" s="2"/>
       <c r="H153" s="2"/>
@@ -65189,8 +65199,8 @@
       </c>
       <c r="B154" s="334"/>
       <c r="C154" s="71"/>
-      <c r="D154" s="457"/>
-      <c r="E154" s="392"/>
+      <c r="D154" s="456"/>
+      <c r="E154" s="393"/>
       <c r="F154" s="2"/>
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
@@ -65204,8 +65214,8 @@
       </c>
       <c r="B155" s="334"/>
       <c r="C155" s="71"/>
-      <c r="D155" s="454"/>
-      <c r="E155" s="392"/>
+      <c r="D155" s="446"/>
+      <c r="E155" s="393"/>
       <c r="F155" s="2"/>
       <c r="G155" s="2"/>
       <c r="H155" s="2"/>
@@ -65219,8 +65229,8 @@
       </c>
       <c r="B156" s="334"/>
       <c r="C156" s="71"/>
-      <c r="D156" s="454"/>
-      <c r="E156" s="392"/>
+      <c r="D156" s="446"/>
+      <c r="E156" s="393"/>
       <c r="F156" s="2"/>
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
@@ -65234,8 +65244,8 @@
       </c>
       <c r="B157" s="7"/>
       <c r="C157" s="333"/>
-      <c r="D157" s="454"/>
-      <c r="E157" s="392"/>
+      <c r="D157" s="446"/>
+      <c r="E157" s="393"/>
       <c r="F157" s="2"/>
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
@@ -65249,8 +65259,8 @@
       </c>
       <c r="B158" s="334"/>
       <c r="C158" s="71"/>
-      <c r="D158" s="454"/>
-      <c r="E158" s="392"/>
+      <c r="D158" s="446"/>
+      <c r="E158" s="393"/>
       <c r="F158" s="2"/>
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
@@ -76206,6 +76216,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A54:K54"/>
+    <mergeCell ref="A87:K87"/>
+    <mergeCell ref="A121:K121"/>
     <mergeCell ref="A141:F141"/>
     <mergeCell ref="D143:E143"/>
     <mergeCell ref="D157:E157"/>
@@ -76217,11 +76232,6 @@
     <mergeCell ref="D154:E154"/>
     <mergeCell ref="D155:E155"/>
     <mergeCell ref="D156:E156"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A36:K36"/>
-    <mergeCell ref="A54:K54"/>
-    <mergeCell ref="A87:K87"/>
-    <mergeCell ref="A121:K121"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: support historical unfinished teacher sessions
</commit_message>
<xml_diff>
--- a/yazokulu.xlsx
+++ b/yazokulu.xlsx
@@ -5276,7 +5276,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -5461,11 +5461,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="460">
+  <cellXfs count="468">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6535,26 +6550,29 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6566,10 +6584,10 @@
     <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="25" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6581,25 +6599,22 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6620,6 +6635,12 @@
     <xf numFmtId="0" fontId="33" fillId="27" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="37" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6629,14 +6650,26 @@
     <xf numFmtId="0" fontId="4" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -6650,24 +6683,6 @@
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -6680,6 +6695,18 @@
     <xf numFmtId="0" fontId="38" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -32576,7 +32603,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="100.5" customHeight="1">
       <c r="A1" s="210"/>
-      <c r="B1" s="429" t="s">
+      <c r="B1" s="417" t="s">
         <v>326</v>
       </c>
       <c r="C1" s="392"/>
@@ -32595,7 +32622,7 @@
     </row>
     <row r="2" spans="1:17" ht="38.25" customHeight="1">
       <c r="A2" s="211"/>
-      <c r="B2" s="430" t="s">
+      <c r="B2" s="418" t="s">
         <v>291</v>
       </c>
       <c r="C2" s="392"/>
@@ -32614,58 +32641,58 @@
     </row>
     <row r="3" spans="1:17" ht="14.4">
       <c r="A3" s="34"/>
-      <c r="B3" s="422" t="s">
+      <c r="B3" s="419" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="179">
         <v>108</v>
       </c>
       <c r="D3" s="179"/>
-      <c r="E3" s="411" t="s">
+      <c r="E3" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="F3" s="422" t="s">
+      <c r="F3" s="419" t="s">
         <v>3</v>
       </c>
       <c r="G3" s="179">
         <v>105</v>
       </c>
       <c r="H3" s="179"/>
-      <c r="I3" s="411" t="s">
+      <c r="I3" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="J3" s="422" t="s">
+      <c r="J3" s="419" t="s">
         <v>5</v>
       </c>
       <c r="K3" s="179">
         <v>103</v>
       </c>
       <c r="L3" s="179"/>
-      <c r="M3" s="411" t="s">
+      <c r="M3" s="412" t="s">
         <v>327</v>
       </c>
       <c r="Q3" s="35"/>
     </row>
     <row r="4" spans="1:17" ht="14.4">
       <c r="A4" s="34"/>
-      <c r="B4" s="412"/>
+      <c r="B4" s="411"/>
       <c r="C4" s="179" t="s">
         <v>328</v>
       </c>
       <c r="D4" s="179"/>
-      <c r="E4" s="412"/>
-      <c r="F4" s="412"/>
+      <c r="E4" s="411"/>
+      <c r="F4" s="411"/>
       <c r="G4" s="179" t="s">
         <v>220</v>
       </c>
       <c r="H4" s="179"/>
-      <c r="I4" s="412"/>
-      <c r="J4" s="412"/>
+      <c r="I4" s="411"/>
+      <c r="J4" s="411"/>
       <c r="K4" s="179" t="s">
         <v>329</v>
       </c>
       <c r="L4" s="179"/>
-      <c r="M4" s="412"/>
+      <c r="M4" s="411"/>
       <c r="Q4" s="35"/>
     </row>
     <row r="5" spans="1:17" ht="22.5" customHeight="1">
@@ -33113,30 +33140,30 @@
     </row>
     <row r="19" spans="1:17" ht="14.4">
       <c r="A19" s="34"/>
-      <c r="B19" s="422" t="s">
+      <c r="B19" s="419" t="s">
         <v>68</v>
       </c>
       <c r="C19" s="179">
         <v>107</v>
       </c>
       <c r="D19" s="179"/>
-      <c r="E19" s="411" t="s">
+      <c r="E19" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="F19" s="425" t="s">
+      <c r="F19" s="426" t="s">
         <v>68</v>
       </c>
       <c r="G19" s="216">
         <v>106</v>
       </c>
       <c r="H19" s="217"/>
-      <c r="I19" s="426" t="s">
+      <c r="I19" s="427" t="s">
         <v>327</v>
       </c>
-      <c r="J19" s="416"/>
-      <c r="K19" s="427"/>
+      <c r="J19" s="428"/>
+      <c r="K19" s="429"/>
       <c r="L19" s="400"/>
-      <c r="M19" s="419"/>
+      <c r="M19" s="420"/>
       <c r="N19" s="35"/>
       <c r="O19" s="35"/>
       <c r="P19" s="35"/>
@@ -33144,18 +33171,18 @@
     </row>
     <row r="20" spans="1:17" ht="21.75" customHeight="1">
       <c r="A20" s="34"/>
-      <c r="B20" s="412"/>
+      <c r="B20" s="411"/>
       <c r="C20" s="179" t="s">
         <v>343</v>
       </c>
       <c r="D20" s="179"/>
-      <c r="E20" s="412"/>
-      <c r="F20" s="412"/>
+      <c r="E20" s="411"/>
+      <c r="F20" s="411"/>
       <c r="G20" s="218" t="s">
         <v>344</v>
       </c>
       <c r="H20" s="217"/>
-      <c r="I20" s="412"/>
+      <c r="I20" s="411"/>
       <c r="J20" s="400"/>
       <c r="K20" s="400"/>
       <c r="L20" s="400"/>
@@ -33221,7 +33248,7 @@
       <c r="L22" s="48"/>
       <c r="M22" s="9"/>
       <c r="N22" s="224"/>
-      <c r="O22" s="420"/>
+      <c r="O22" s="421"/>
       <c r="Q22" s="35"/>
     </row>
     <row r="23" spans="1:17" ht="14.4">
@@ -33560,7 +33587,7 @@
     </row>
     <row r="35" spans="1:17" ht="30.75" customHeight="1">
       <c r="A35" s="211"/>
-      <c r="B35" s="428" t="s">
+      <c r="B35" s="430" t="s">
         <v>297</v>
       </c>
       <c r="C35" s="392"/>
@@ -33588,17 +33615,17 @@
         <v>105</v>
       </c>
       <c r="D36" s="231"/>
-      <c r="E36" s="411" t="s">
+      <c r="E36" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="F36" s="415" t="s">
+      <c r="F36" s="431" t="s">
         <v>5</v>
       </c>
       <c r="G36" s="232">
         <v>107</v>
       </c>
       <c r="H36" s="231"/>
-      <c r="I36" s="411" t="s">
+      <c r="I36" s="412" t="s">
         <v>327</v>
       </c>
       <c r="J36" s="34"/>
@@ -33609,18 +33636,18 @@
     </row>
     <row r="37" spans="1:17" ht="21.75" customHeight="1">
       <c r="A37" s="47"/>
-      <c r="B37" s="412"/>
+      <c r="B37" s="411"/>
       <c r="C37" s="231" t="s">
         <v>352</v>
       </c>
       <c r="D37" s="231"/>
-      <c r="E37" s="412"/>
-      <c r="F37" s="412"/>
+      <c r="E37" s="411"/>
+      <c r="F37" s="411"/>
       <c r="G37" s="231" t="s">
         <v>343</v>
       </c>
       <c r="H37" s="231"/>
-      <c r="I37" s="412"/>
+      <c r="I37" s="411"/>
       <c r="J37" s="34"/>
       <c r="K37" s="34"/>
       <c r="L37" s="34"/>
@@ -33676,7 +33703,7 @@
       <c r="I39" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="J39" s="416"/>
+      <c r="J39" s="428"/>
       <c r="K39" s="400"/>
       <c r="L39" s="400"/>
       <c r="M39" s="35"/>
@@ -33769,7 +33796,7 @@
       <c r="I42" s="185" t="s">
         <v>224</v>
       </c>
-      <c r="J42" s="416"/>
+      <c r="J42" s="428"/>
       <c r="K42" s="400"/>
       <c r="L42" s="400"/>
       <c r="M42" s="35"/>
@@ -34026,7 +34053,7 @@
     </row>
     <row r="53" spans="1:17" ht="25.5" customHeight="1">
       <c r="A53" s="211"/>
-      <c r="B53" s="417" t="s">
+      <c r="B53" s="432" t="s">
         <v>363</v>
       </c>
       <c r="C53" s="392"/>
@@ -34043,58 +34070,58 @@
     </row>
     <row r="54" spans="1:17" ht="20.25" customHeight="1">
       <c r="A54" s="34"/>
-      <c r="B54" s="418" t="s">
+      <c r="B54" s="424" t="s">
         <v>3</v>
       </c>
       <c r="C54" s="195" t="s">
         <v>329</v>
       </c>
       <c r="D54" s="195"/>
-      <c r="E54" s="411" t="s">
+      <c r="E54" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="F54" s="418" t="s">
+      <c r="F54" s="424" t="s">
         <v>5</v>
       </c>
       <c r="G54" s="238" t="s">
         <v>328</v>
       </c>
       <c r="H54" s="195"/>
-      <c r="I54" s="411" t="s">
+      <c r="I54" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="J54" s="418" t="s">
+      <c r="J54" s="424" t="s">
         <v>68</v>
       </c>
       <c r="K54" s="195" t="s">
         <v>220</v>
       </c>
       <c r="L54" s="239"/>
-      <c r="M54" s="411" t="s">
+      <c r="M54" s="412" t="s">
         <v>327</v>
       </c>
       <c r="Q54" s="35"/>
     </row>
     <row r="55" spans="1:17" ht="20.25" customHeight="1">
       <c r="A55" s="34"/>
-      <c r="B55" s="412"/>
+      <c r="B55" s="411"/>
       <c r="C55" s="195">
         <v>105</v>
       </c>
       <c r="D55" s="195"/>
-      <c r="E55" s="412"/>
-      <c r="F55" s="412"/>
+      <c r="E55" s="411"/>
+      <c r="F55" s="411"/>
       <c r="G55" s="240">
         <v>108</v>
       </c>
       <c r="H55" s="195"/>
-      <c r="I55" s="412"/>
-      <c r="J55" s="412"/>
+      <c r="I55" s="411"/>
+      <c r="J55" s="411"/>
       <c r="K55" s="195">
         <v>106</v>
       </c>
       <c r="L55" s="239"/>
-      <c r="M55" s="412"/>
+      <c r="M55" s="411"/>
       <c r="Q55" s="35"/>
     </row>
     <row r="56" spans="1:17" ht="23.25" customHeight="1">
@@ -34574,7 +34601,7 @@
     </row>
     <row r="72" spans="1:19" ht="24" customHeight="1">
       <c r="A72" s="211"/>
-      <c r="B72" s="413" t="s">
+      <c r="B72" s="433" t="s">
         <v>300</v>
       </c>
       <c r="C72" s="392"/>
@@ -34592,34 +34619,34 @@
     </row>
     <row r="73" spans="1:19" ht="21.75" customHeight="1">
       <c r="A73" s="34"/>
-      <c r="B73" s="424" t="s">
+      <c r="B73" s="425" t="s">
         <v>0</v>
       </c>
       <c r="C73" s="248" t="s">
         <v>328</v>
       </c>
       <c r="D73" s="248"/>
-      <c r="E73" s="411" t="s">
+      <c r="E73" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="F73" s="414" t="s">
+      <c r="F73" s="413" t="s">
         <v>5</v>
       </c>
       <c r="G73" s="206" t="s">
         <v>370</v>
       </c>
       <c r="H73" s="206"/>
-      <c r="I73" s="411" t="s">
+      <c r="I73" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="J73" s="414" t="s">
+      <c r="J73" s="413" t="s">
         <v>68</v>
       </c>
       <c r="K73" s="72" t="s">
         <v>329</v>
       </c>
       <c r="L73" s="72"/>
-      <c r="M73" s="411" t="s">
+      <c r="M73" s="412" t="s">
         <v>327</v>
       </c>
       <c r="N73" s="34"/>
@@ -34631,24 +34658,24 @@
     </row>
     <row r="74" spans="1:19" ht="21.75" customHeight="1">
       <c r="A74" s="34"/>
-      <c r="B74" s="412"/>
+      <c r="B74" s="411"/>
       <c r="C74" s="248">
         <v>108</v>
       </c>
       <c r="D74" s="248"/>
-      <c r="E74" s="412"/>
-      <c r="F74" s="412"/>
+      <c r="E74" s="411"/>
+      <c r="F74" s="411"/>
       <c r="G74" s="206">
         <v>106</v>
       </c>
       <c r="H74" s="206"/>
-      <c r="I74" s="412"/>
-      <c r="J74" s="412"/>
+      <c r="I74" s="411"/>
+      <c r="J74" s="411"/>
       <c r="K74" s="72">
         <v>105</v>
       </c>
       <c r="L74" s="72"/>
-      <c r="M74" s="412"/>
+      <c r="M74" s="411"/>
       <c r="N74" s="34"/>
       <c r="O74" s="34"/>
       <c r="P74" s="34"/>
@@ -35249,58 +35276,58 @@
     </row>
     <row r="90" spans="1:19" ht="14.4">
       <c r="A90" s="34"/>
-      <c r="B90" s="414" t="s">
+      <c r="B90" s="413" t="s">
         <v>243</v>
       </c>
       <c r="C90" s="72" t="s">
         <v>220</v>
       </c>
       <c r="D90" s="72"/>
-      <c r="E90" s="411" t="s">
+      <c r="E90" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="F90" s="414" t="s">
+      <c r="F90" s="413" t="s">
         <v>48</v>
       </c>
       <c r="G90" s="72" t="s">
         <v>386</v>
       </c>
       <c r="H90" s="72"/>
-      <c r="I90" s="411" t="s">
+      <c r="I90" s="412" t="s">
         <v>327</v>
       </c>
-      <c r="J90" s="431" t="s">
+      <c r="J90" s="414" t="s">
         <v>135</v>
       </c>
       <c r="K90" s="72" t="s">
         <v>387</v>
       </c>
       <c r="L90" s="72"/>
-      <c r="M90" s="432" t="s">
+      <c r="M90" s="415" t="s">
         <v>327</v>
       </c>
       <c r="Q90" s="35"/>
     </row>
     <row r="91" spans="1:19" ht="14.4">
       <c r="A91" s="34"/>
-      <c r="B91" s="412"/>
+      <c r="B91" s="411"/>
       <c r="C91" s="72">
         <v>104</v>
       </c>
       <c r="D91" s="72"/>
-      <c r="E91" s="412"/>
-      <c r="F91" s="412"/>
+      <c r="E91" s="411"/>
+      <c r="F91" s="411"/>
       <c r="G91" s="72">
         <v>107</v>
       </c>
       <c r="H91" s="72"/>
-      <c r="I91" s="412"/>
-      <c r="J91" s="412"/>
+      <c r="I91" s="411"/>
+      <c r="J91" s="411"/>
       <c r="K91" s="72">
         <v>103</v>
       </c>
       <c r="L91" s="72"/>
-      <c r="M91" s="412"/>
+      <c r="M91" s="411"/>
       <c r="Q91" s="35"/>
     </row>
     <row r="92" spans="1:19" ht="24" customHeight="1">
@@ -35788,7 +35815,7 @@
     </row>
     <row r="107" spans="1:27" ht="21">
       <c r="A107" s="58"/>
-      <c r="B107" s="433" t="s">
+      <c r="B107" s="416" t="s">
         <v>302</v>
       </c>
       <c r="C107" s="407"/>
@@ -35812,39 +35839,39 @@
         <v>352</v>
       </c>
       <c r="D108" s="168"/>
-      <c r="E108" s="411" t="s">
+      <c r="E108" s="412" t="s">
         <v>327</v>
       </c>
       <c r="F108" s="401"/>
       <c r="G108" s="168"/>
       <c r="H108" s="168"/>
-      <c r="I108" s="411" t="s">
+      <c r="I108" s="412" t="s">
         <v>398</v>
       </c>
       <c r="J108" s="401"/>
       <c r="K108" s="168"/>
       <c r="L108" s="168"/>
-      <c r="M108" s="411" t="s">
+      <c r="M108" s="412" t="s">
         <v>327</v>
       </c>
       <c r="Q108" s="35"/>
     </row>
     <row r="109" spans="1:27" ht="14.4">
       <c r="A109" s="47"/>
-      <c r="B109" s="412"/>
+      <c r="B109" s="411"/>
       <c r="C109" s="168">
         <v>106</v>
       </c>
       <c r="D109" s="168"/>
-      <c r="E109" s="412"/>
-      <c r="F109" s="412"/>
+      <c r="E109" s="411"/>
+      <c r="F109" s="411"/>
       <c r="G109" s="168"/>
       <c r="H109" s="168"/>
-      <c r="I109" s="412"/>
-      <c r="J109" s="412"/>
+      <c r="I109" s="411"/>
+      <c r="J109" s="411"/>
       <c r="K109" s="168"/>
       <c r="L109" s="168"/>
-      <c r="M109" s="412"/>
+      <c r="M109" s="411"/>
       <c r="Q109" s="35"/>
     </row>
     <row r="110" spans="1:27" ht="22.5" customHeight="1">
@@ -35901,7 +35928,7 @@
       <c r="K111" s="98"/>
       <c r="L111" s="12"/>
       <c r="M111" s="45"/>
-      <c r="N111" s="421"/>
+      <c r="N111" s="422"/>
       <c r="O111" s="400"/>
       <c r="Q111" s="35"/>
     </row>
@@ -38980,25 +39007,22 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="F108:F110"/>
-    <mergeCell ref="I108:I110"/>
-    <mergeCell ref="J108:J110"/>
-    <mergeCell ref="M108:M110"/>
-    <mergeCell ref="E90:E92"/>
-    <mergeCell ref="F90:F92"/>
-    <mergeCell ref="I90:I92"/>
-    <mergeCell ref="J90:J92"/>
-    <mergeCell ref="M90:M92"/>
-    <mergeCell ref="B107:L107"/>
-    <mergeCell ref="E108:E110"/>
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="F3:F5"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="M3:M5"/>
-    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="M73:M75"/>
+    <mergeCell ref="B72:L72"/>
+    <mergeCell ref="E73:E75"/>
+    <mergeCell ref="F73:F75"/>
+    <mergeCell ref="I73:I75"/>
+    <mergeCell ref="J73:J75"/>
+    <mergeCell ref="I54:I56"/>
+    <mergeCell ref="M54:M56"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="F36:F38"/>
+    <mergeCell ref="I36:I38"/>
+    <mergeCell ref="J39:L41"/>
+    <mergeCell ref="J42:L44"/>
+    <mergeCell ref="B53:L53"/>
+    <mergeCell ref="E54:E56"/>
+    <mergeCell ref="J54:J56"/>
     <mergeCell ref="M19:M21"/>
     <mergeCell ref="O22:O25"/>
     <mergeCell ref="N111:O115"/>
@@ -39015,22 +39039,25 @@
     <mergeCell ref="K19:L20"/>
     <mergeCell ref="B35:L35"/>
     <mergeCell ref="F54:F56"/>
-    <mergeCell ref="I54:I56"/>
-    <mergeCell ref="M54:M56"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="F36:F38"/>
-    <mergeCell ref="I36:I38"/>
-    <mergeCell ref="J39:L41"/>
-    <mergeCell ref="J42:L44"/>
-    <mergeCell ref="B53:L53"/>
-    <mergeCell ref="E54:E56"/>
-    <mergeCell ref="J54:J56"/>
-    <mergeCell ref="M73:M75"/>
-    <mergeCell ref="B72:L72"/>
-    <mergeCell ref="E73:E75"/>
-    <mergeCell ref="F73:F75"/>
-    <mergeCell ref="I73:I75"/>
-    <mergeCell ref="J73:J75"/>
+    <mergeCell ref="B1:N1"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="F3:F5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="M3:M5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="F108:F110"/>
+    <mergeCell ref="I108:I110"/>
+    <mergeCell ref="J108:J110"/>
+    <mergeCell ref="M108:M110"/>
+    <mergeCell ref="E90:E92"/>
+    <mergeCell ref="F90:F92"/>
+    <mergeCell ref="I90:I92"/>
+    <mergeCell ref="J90:J92"/>
+    <mergeCell ref="M90:M92"/>
+    <mergeCell ref="B107:L107"/>
+    <mergeCell ref="E108:E110"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -39066,14 +39093,14 @@
       <c r="G1" s="400"/>
     </row>
     <row r="2" spans="1:8" ht="14.4">
-      <c r="A2" s="422" t="s">
+      <c r="A2" s="419" t="s">
         <v>480</v>
       </c>
       <c r="B2" s="179" t="s">
         <v>344</v>
       </c>
       <c r="C2" s="179"/>
-      <c r="E2" s="422" t="s">
+      <c r="E2" s="419" t="s">
         <v>481</v>
       </c>
       <c r="F2" s="179" t="s">
@@ -39082,14 +39109,14 @@
       <c r="G2" s="179"/>
     </row>
     <row r="3" spans="1:8" ht="14.4">
-      <c r="A3" s="412"/>
+      <c r="A3" s="411"/>
       <c r="B3" s="179">
         <v>108</v>
       </c>
       <c r="C3" s="179" t="s">
         <v>482</v>
       </c>
-      <c r="E3" s="412"/>
+      <c r="E3" s="411"/>
       <c r="F3" s="179">
         <v>107</v>
       </c>
@@ -39977,13 +40004,13 @@
         <v>9</v>
       </c>
       <c r="F15" s="273" t="s">
-        <v>434</v>
+        <v>455</v>
       </c>
       <c r="G15" s="272">
         <v>2017</v>
       </c>
       <c r="H15" s="185">
-        <v>5395823847</v>
+        <v>5396152431</v>
       </c>
       <c r="I15" s="273">
         <v>9</v>
@@ -40015,13 +40042,13 @@
         <v>10</v>
       </c>
       <c r="F16" s="273" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="G16" s="272">
         <v>2017</v>
       </c>
       <c r="H16" s="185">
-        <v>5396152431</v>
+        <v>5384327013</v>
       </c>
       <c r="I16" s="273">
         <v>10</v>
@@ -40049,17 +40076,17 @@
       <c r="D17" s="45">
         <v>5358268513</v>
       </c>
-      <c r="E17" s="45">
+      <c r="E17" s="462">
         <v>11</v>
       </c>
-      <c r="F17" s="273" t="s">
-        <v>456</v>
-      </c>
-      <c r="G17" s="272">
-        <v>2017</v>
-      </c>
-      <c r="H17" s="185">
-        <v>5384327013</v>
+      <c r="F17" s="463" t="s">
+        <v>451</v>
+      </c>
+      <c r="G17" s="464">
+        <v>2019</v>
+      </c>
+      <c r="H17" s="465">
+        <v>5425771950</v>
       </c>
       <c r="I17" s="273">
         <v>11</v>
@@ -40084,22 +40111,14 @@
       <c r="C18" s="269">
         <v>2014</v>
       </c>
-      <c r="D18" s="45">
+      <c r="D18" s="460">
         <v>5435322375</v>
       </c>
-      <c r="E18" s="45">
-        <v>12</v>
-      </c>
-      <c r="F18" s="287" t="s">
-        <v>451</v>
-      </c>
-      <c r="G18" s="288">
-        <v>2019</v>
-      </c>
-      <c r="H18" s="185">
-        <v>5425771950</v>
-      </c>
-      <c r="I18" s="273">
+      <c r="E18" s="467"/>
+      <c r="F18" s="467"/>
+      <c r="G18" s="467"/>
+      <c r="H18" s="467"/>
+      <c r="I18" s="461">
         <v>12</v>
       </c>
       <c r="J18" s="294" t="s">
@@ -40113,7 +40132,7 @@
       </c>
     </row>
     <row r="19" spans="1:16" ht="17.399999999999999">
-      <c r="E19" s="45"/>
+      <c r="E19" s="466"/>
       <c r="I19" s="274"/>
       <c r="J19" s="32"/>
       <c r="K19" s="32"/>
@@ -40829,7 +40848,19 @@
         <v>5307978853</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="14.4">
+    <row r="37" spans="1:16" ht="18">
+      <c r="A37" s="45">
+        <v>13</v>
+      </c>
+      <c r="B37" s="273" t="s">
+        <v>434</v>
+      </c>
+      <c r="C37" s="272">
+        <v>2017</v>
+      </c>
+      <c r="D37" s="185">
+        <v>5395823847</v>
+      </c>
       <c r="E37" s="6"/>
       <c r="M37" s="35"/>
       <c r="N37" s="35"/>
@@ -40923,7 +40954,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="33" customHeight="1">
-      <c r="A1" s="440" t="s">
+      <c r="A1" s="442" t="s">
         <v>532</v>
       </c>
       <c r="B1" s="400"/>
@@ -40941,7 +40972,7 @@
       <c r="N1" s="35"/>
     </row>
     <row r="2" spans="1:14" ht="33" customHeight="1">
-      <c r="A2" s="441" t="s">
+      <c r="A2" s="443" t="s">
         <v>533</v>
       </c>
       <c r="B2" s="392"/>
@@ -40959,34 +40990,34 @@
       <c r="N2" s="35"/>
     </row>
     <row r="3" spans="1:14" ht="15.6">
-      <c r="A3" s="422"/>
+      <c r="A3" s="419"/>
       <c r="B3" s="305" t="s">
         <v>534</v>
       </c>
       <c r="C3" s="179"/>
-      <c r="D3" s="411"/>
-      <c r="E3" s="442"/>
+      <c r="D3" s="412"/>
+      <c r="E3" s="444"/>
       <c r="F3" s="306" t="s">
         <v>535</v>
       </c>
       <c r="G3" s="137"/>
-      <c r="H3" s="411"/>
-      <c r="I3" s="416"/>
+      <c r="H3" s="412"/>
+      <c r="I3" s="428"/>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
-      <c r="L3" s="419"/>
+      <c r="L3" s="420"/>
       <c r="M3" s="35"/>
       <c r="N3" s="35"/>
     </row>
     <row r="4" spans="1:14" ht="14.4">
-      <c r="A4" s="412"/>
+      <c r="A4" s="411"/>
       <c r="B4" s="179"/>
       <c r="C4" s="179"/>
-      <c r="D4" s="412"/>
-      <c r="E4" s="412"/>
+      <c r="D4" s="411"/>
+      <c r="E4" s="411"/>
       <c r="F4" s="137"/>
       <c r="G4" s="137"/>
-      <c r="H4" s="412"/>
+      <c r="H4" s="411"/>
       <c r="I4" s="400"/>
       <c r="J4" s="34"/>
       <c r="K4" s="34"/>
@@ -41305,7 +41336,7 @@
       </c>
     </row>
     <row r="20" spans="1:12" ht="26.25" customHeight="1">
-      <c r="A20" s="428" t="s">
+      <c r="A20" s="430" t="s">
         <v>551</v>
       </c>
       <c r="B20" s="392"/>
@@ -41321,30 +41352,30 @@
       <c r="L20" s="35"/>
     </row>
     <row r="21" spans="1:12" ht="14.4">
-      <c r="A21" s="443"/>
+      <c r="A21" s="440"/>
       <c r="B21" s="310" t="s">
         <v>552</v>
       </c>
       <c r="C21" s="310"/>
-      <c r="D21" s="411"/>
-      <c r="E21" s="444"/>
+      <c r="D21" s="412"/>
+      <c r="E21" s="441"/>
       <c r="F21" s="148"/>
       <c r="G21" s="148"/>
-      <c r="H21" s="411"/>
+      <c r="H21" s="412"/>
       <c r="I21" s="34"/>
       <c r="J21" s="34"/>
       <c r="K21" s="34"/>
       <c r="L21" s="35"/>
     </row>
     <row r="22" spans="1:12" ht="14.4">
-      <c r="A22" s="412"/>
+      <c r="A22" s="411"/>
       <c r="B22" s="310"/>
       <c r="C22" s="310"/>
-      <c r="D22" s="412"/>
-      <c r="E22" s="412"/>
+      <c r="D22" s="411"/>
+      <c r="E22" s="411"/>
       <c r="F22" s="148"/>
       <c r="G22" s="148"/>
-      <c r="H22" s="412"/>
+      <c r="H22" s="411"/>
       <c r="I22" s="34"/>
       <c r="J22" s="34"/>
       <c r="K22" s="34"/>
@@ -41672,11 +41703,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="L3:L5"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:H2"/>
@@ -41685,6 +41711,11 @@
     <mergeCell ref="E3:E5"/>
     <mergeCell ref="I3:I5"/>
     <mergeCell ref="H3:H5"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="H21:H23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -41726,7 +41757,7 @@
     </row>
     <row r="2" spans="1:16" ht="21">
       <c r="A2" s="2"/>
-      <c r="B2" s="454" t="s">
+      <c r="B2" s="445" t="s">
         <v>567</v>
       </c>
       <c r="C2" s="392"/>
@@ -41742,13 +41773,13 @@
     </row>
     <row r="3" spans="1:16" ht="14.4">
       <c r="A3" s="2"/>
-      <c r="B3" s="452" t="s">
+      <c r="B3" s="446" t="s">
         <v>568</v>
       </c>
       <c r="C3" s="400"/>
       <c r="D3" s="400"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="445" t="s">
+      <c r="F3" s="447" t="s">
         <v>568</v>
       </c>
       <c r="G3" s="392"/>
@@ -42092,13 +42123,13 @@
     </row>
     <row r="19" spans="1:9" ht="14.4">
       <c r="A19" s="2"/>
-      <c r="B19" s="455" t="s">
+      <c r="B19" s="448" t="s">
         <v>568</v>
       </c>
       <c r="C19" s="407"/>
       <c r="D19" s="408"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="445" t="s">
+      <c r="F19" s="447" t="s">
         <v>568</v>
       </c>
       <c r="G19" s="392"/>
@@ -42409,7 +42440,7 @@
     </row>
     <row r="34" spans="1:12" ht="15.75" customHeight="1">
       <c r="A34" s="2"/>
-      <c r="B34" s="451" t="s">
+      <c r="B34" s="449" t="s">
         <v>599</v>
       </c>
       <c r="C34" s="392"/>
@@ -42425,13 +42456,13 @@
     </row>
     <row r="35" spans="1:12" ht="15.75" customHeight="1">
       <c r="A35" s="2"/>
-      <c r="B35" s="445" t="s">
+      <c r="B35" s="447" t="s">
         <v>568</v>
       </c>
       <c r="C35" s="392"/>
       <c r="D35" s="393"/>
       <c r="E35" s="2"/>
-      <c r="F35" s="452" t="s">
+      <c r="F35" s="446" t="s">
         <v>568</v>
       </c>
       <c r="G35" s="400"/>
@@ -42812,7 +42843,7 @@
     </row>
     <row r="52" spans="1:12" ht="20.25" customHeight="1">
       <c r="A52" s="2"/>
-      <c r="B52" s="453" t="s">
+      <c r="B52" s="450" t="s">
         <v>615</v>
       </c>
       <c r="C52" s="392"/>
@@ -42828,13 +42859,13 @@
     </row>
     <row r="53" spans="1:12" ht="20.25" customHeight="1">
       <c r="A53" s="2"/>
-      <c r="B53" s="445" t="s">
+      <c r="B53" s="447" t="s">
         <v>568</v>
       </c>
       <c r="C53" s="392"/>
       <c r="D53" s="393"/>
       <c r="E53" s="2"/>
-      <c r="F53" s="445" t="s">
+      <c r="F53" s="447" t="s">
         <v>568</v>
       </c>
       <c r="G53" s="392"/>
@@ -43258,19 +43289,19 @@
     </row>
     <row r="69" spans="1:12" ht="15.75" customHeight="1">
       <c r="A69" s="2"/>
-      <c r="B69" s="445" t="s">
+      <c r="B69" s="447" t="s">
         <v>568</v>
       </c>
       <c r="C69" s="392"/>
       <c r="D69" s="393"/>
       <c r="E69" s="2"/>
-      <c r="F69" s="445" t="s">
+      <c r="F69" s="447" t="s">
         <v>568</v>
       </c>
       <c r="G69" s="392"/>
       <c r="H69" s="393"/>
       <c r="I69" s="2"/>
-      <c r="J69" s="445" t="s">
+      <c r="J69" s="447" t="s">
         <v>568</v>
       </c>
       <c r="K69" s="392"/>
@@ -43664,7 +43695,7 @@
     </row>
     <row r="85" spans="1:12" ht="15.75" customHeight="1">
       <c r="A85" s="2"/>
-      <c r="B85" s="450" t="s">
+      <c r="B85" s="451" t="s">
         <v>645</v>
       </c>
       <c r="C85" s="392"/>
@@ -43680,19 +43711,19 @@
     </row>
     <row r="86" spans="1:12" ht="15.75" customHeight="1">
       <c r="A86" s="2"/>
-      <c r="B86" s="445" t="s">
+      <c r="B86" s="447" t="s">
         <v>568</v>
       </c>
       <c r="C86" s="392"/>
       <c r="D86" s="393"/>
       <c r="E86" s="2"/>
-      <c r="F86" s="445" t="s">
+      <c r="F86" s="447" t="s">
         <v>568</v>
       </c>
       <c r="G86" s="392"/>
       <c r="H86" s="393"/>
       <c r="I86" s="2"/>
-      <c r="J86" s="445" t="s">
+      <c r="J86" s="447" t="s">
         <v>568</v>
       </c>
       <c r="K86" s="392"/>
@@ -44181,19 +44212,19 @@
     </row>
     <row r="103" spans="1:13" ht="15.75" customHeight="1">
       <c r="A103" s="2"/>
-      <c r="B103" s="445" t="s">
+      <c r="B103" s="447" t="s">
         <v>568</v>
       </c>
       <c r="C103" s="392"/>
       <c r="D103" s="393"/>
       <c r="E103" s="2"/>
-      <c r="F103" s="445" t="s">
+      <c r="F103" s="447" t="s">
         <v>568</v>
       </c>
       <c r="G103" s="392"/>
       <c r="H103" s="393"/>
       <c r="I103" s="2"/>
-      <c r="J103" s="445" t="s">
+      <c r="J103" s="447" t="s">
         <v>568</v>
       </c>
       <c r="K103" s="392"/>
@@ -44644,7 +44675,7 @@
     </row>
     <row r="119" spans="1:12" ht="15.75" customHeight="1">
       <c r="A119" s="2"/>
-      <c r="B119" s="445" t="s">
+      <c r="B119" s="447" t="s">
         <v>568</v>
       </c>
       <c r="C119" s="392"/>
@@ -44938,7 +44969,7 @@
     </row>
     <row r="135" spans="1:13" ht="15.75" customHeight="1">
       <c r="A135" s="2"/>
-      <c r="B135" s="447" t="s">
+      <c r="B135" s="453" t="s">
         <v>697</v>
       </c>
       <c r="C135" s="392"/>
@@ -44954,19 +44985,19 @@
     </row>
     <row r="136" spans="1:13" ht="15.75" customHeight="1">
       <c r="A136" s="2"/>
-      <c r="B136" s="445" t="s">
+      <c r="B136" s="447" t="s">
         <v>568</v>
       </c>
       <c r="C136" s="392"/>
       <c r="D136" s="393"/>
       <c r="E136" s="2"/>
-      <c r="F136" s="445" t="s">
+      <c r="F136" s="447" t="s">
         <v>568</v>
       </c>
       <c r="G136" s="392"/>
       <c r="H136" s="393"/>
       <c r="I136" s="2"/>
-      <c r="J136" s="445" t="s">
+      <c r="J136" s="447" t="s">
         <v>568</v>
       </c>
       <c r="K136" s="392"/>
@@ -45463,7 +45494,7 @@
     </row>
     <row r="155" spans="1:12" ht="15.75" customHeight="1">
       <c r="A155" s="2"/>
-      <c r="B155" s="448" t="s">
+      <c r="B155" s="454" t="s">
         <v>722</v>
       </c>
       <c r="C155" s="392"/>
@@ -45500,7 +45531,7 @@
       <c r="D157" s="346" t="s">
         <v>8</v>
       </c>
-      <c r="E157" s="449" t="s">
+      <c r="E157" s="455" t="s">
         <v>723</v>
       </c>
       <c r="F157" s="393"/>
@@ -45544,7 +45575,7 @@
       <c r="D159" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="E159" s="446" t="s">
+      <c r="E159" s="452" t="s">
         <v>727</v>
       </c>
       <c r="F159" s="393"/>
@@ -45650,7 +45681,7 @@
       </c>
       <c r="C164" s="334"/>
       <c r="D164" s="71"/>
-      <c r="E164" s="446"/>
+      <c r="E164" s="452"/>
       <c r="F164" s="393"/>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
@@ -57449,24 +57480,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="B34:L34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="B52:L52"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="F69:H69"/>
-    <mergeCell ref="J69:L69"/>
-    <mergeCell ref="B85:L85"/>
-    <mergeCell ref="B86:D86"/>
-    <mergeCell ref="F86:H86"/>
-    <mergeCell ref="J86:L86"/>
     <mergeCell ref="B103:D103"/>
     <mergeCell ref="F103:H103"/>
     <mergeCell ref="J103:L103"/>
@@ -57479,6 +57492,24 @@
     <mergeCell ref="J136:L136"/>
     <mergeCell ref="B155:G155"/>
     <mergeCell ref="E157:F157"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="F69:H69"/>
+    <mergeCell ref="J69:L69"/>
+    <mergeCell ref="B85:L85"/>
+    <mergeCell ref="B86:D86"/>
+    <mergeCell ref="F86:H86"/>
+    <mergeCell ref="J86:L86"/>
+    <mergeCell ref="B34:L34"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="B52:L52"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="F53:H53"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="F19:H19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -57519,7 +57550,7 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="21">
-      <c r="B2" s="454" t="s">
+      <c r="B2" s="445" t="s">
         <v>736</v>
       </c>
       <c r="C2" s="392"/>
@@ -58180,7 +58211,7 @@
     <row r="34" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="35" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="36" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B36" s="451" t="s">
+      <c r="B36" s="449" t="s">
         <v>599</v>
       </c>
       <c r="C36" s="392"/>
@@ -58439,7 +58470,7 @@
       <c r="L53" s="2"/>
     </row>
     <row r="54" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B54" s="453" t="s">
+      <c r="B54" s="450" t="s">
         <v>615</v>
       </c>
       <c r="C54" s="392"/>
@@ -59194,7 +59225,7 @@
     </row>
     <row r="86" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="87" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B87" s="450" t="s">
+      <c r="B87" s="451" t="s">
         <v>760</v>
       </c>
       <c r="C87" s="392"/>
@@ -60002,7 +60033,7 @@
     <row r="119" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="120" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="121" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B121" s="447" t="s">
+      <c r="B121" s="453" t="s">
         <v>766</v>
       </c>
       <c r="C121" s="392"/>
@@ -60427,7 +60458,7 @@
     <row r="139" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="140" spans="2:12" ht="15.75" customHeight="1"/>
     <row r="141" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B141" s="448" t="s">
+      <c r="B141" s="454" t="s">
         <v>722</v>
       </c>
       <c r="C141" s="392"/>
@@ -60445,7 +60476,7 @@
       <c r="D143" s="346" t="s">
         <v>8</v>
       </c>
-      <c r="E143" s="449" t="s">
+      <c r="E143" s="455" t="s">
         <v>723</v>
       </c>
       <c r="F143" s="393"/>
@@ -60477,7 +60508,7 @@
       <c r="D145" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="E145" s="446" t="s">
+      <c r="E145" s="452" t="s">
         <v>727</v>
       </c>
       <c r="F145" s="393"/>
@@ -60583,7 +60614,7 @@
       <c r="D151" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="E151" s="446"/>
+      <c r="E151" s="452"/>
       <c r="F151" s="393"/>
     </row>
     <row r="152" spans="2:12" ht="15.75" customHeight="1">
@@ -60592,7 +60623,7 @@
       </c>
       <c r="C152" s="7"/>
       <c r="D152" s="71"/>
-      <c r="E152" s="446"/>
+      <c r="E152" s="452"/>
       <c r="F152" s="393"/>
       <c r="G152" s="2"/>
     </row>
@@ -60602,7 +60633,7 @@
       </c>
       <c r="C153" s="71"/>
       <c r="D153" s="71"/>
-      <c r="E153" s="446"/>
+      <c r="E153" s="452"/>
       <c r="F153" s="393"/>
     </row>
     <row r="154" spans="2:12" ht="15.75" customHeight="1">
@@ -60620,7 +60651,7 @@
       </c>
       <c r="C155" s="334"/>
       <c r="D155" s="71"/>
-      <c r="E155" s="446"/>
+      <c r="E155" s="452"/>
       <c r="F155" s="393"/>
     </row>
     <row r="156" spans="2:12" ht="15.75" customHeight="1">
@@ -60629,7 +60660,7 @@
       </c>
       <c r="C156" s="334"/>
       <c r="D156" s="71"/>
-      <c r="E156" s="446"/>
+      <c r="E156" s="452"/>
       <c r="F156" s="393"/>
     </row>
     <row r="157" spans="2:12" ht="15.75" customHeight="1">
@@ -60638,7 +60669,7 @@
       </c>
       <c r="C157" s="7"/>
       <c r="D157" s="333"/>
-      <c r="E157" s="446"/>
+      <c r="E157" s="452"/>
       <c r="F157" s="393"/>
     </row>
     <row r="158" spans="2:12" ht="15.75" customHeight="1">
@@ -60647,7 +60678,7 @@
       </c>
       <c r="C158" s="334"/>
       <c r="D158" s="71"/>
-      <c r="E158" s="446"/>
+      <c r="E158" s="452"/>
       <c r="F158" s="393"/>
     </row>
     <row r="159" spans="2:12" ht="15.75" customHeight="1"/>
@@ -61456,11 +61487,6 @@
     <row r="962" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="B54:L54"/>
-    <mergeCell ref="B87:L87"/>
-    <mergeCell ref="B121:L121"/>
     <mergeCell ref="B141:G141"/>
     <mergeCell ref="E143:F143"/>
     <mergeCell ref="E157:F157"/>
@@ -61472,6 +61498,11 @@
     <mergeCell ref="E154:F154"/>
     <mergeCell ref="E155:F155"/>
     <mergeCell ref="E156:F156"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B54:L54"/>
+    <mergeCell ref="B87:L87"/>
+    <mergeCell ref="B121:L121"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape"/>
@@ -61512,7 +61543,7 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:11" ht="21">
-      <c r="A2" s="454" t="s">
+      <c r="A2" s="445" t="s">
         <v>736</v>
       </c>
       <c r="B2" s="392"/>
@@ -62344,7 +62375,7 @@
       <c r="K35" s="2"/>
     </row>
     <row r="36" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A36" s="451" t="s">
+      <c r="A36" s="449" t="s">
         <v>599</v>
       </c>
       <c r="B36" s="392"/>
@@ -62656,7 +62687,7 @@
       <c r="K53" s="2"/>
     </row>
     <row r="54" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A54" s="453" t="s">
+      <c r="A54" s="450" t="s">
         <v>615</v>
       </c>
       <c r="B54" s="392"/>
@@ -63519,7 +63550,7 @@
       <c r="K86" s="2"/>
     </row>
     <row r="87" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A87" s="450" t="s">
+      <c r="A87" s="451" t="s">
         <v>760</v>
       </c>
       <c r="B87" s="392"/>
@@ -64445,7 +64476,7 @@
       <c r="K120" s="2"/>
     </row>
     <row r="121" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A121" s="447" t="s">
+      <c r="A121" s="453" t="s">
         <v>766</v>
       </c>
       <c r="B121" s="392"/>
@@ -64953,7 +64984,7 @@
       <c r="K140" s="2"/>
     </row>
     <row r="141" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A141" s="448" t="s">
+      <c r="A141" s="454" t="s">
         <v>722</v>
       </c>
       <c r="B141" s="392"/>
@@ -64988,7 +65019,7 @@
       <c r="C143" s="346" t="s">
         <v>8</v>
       </c>
-      <c r="D143" s="449" t="s">
+      <c r="D143" s="455" t="s">
         <v>723</v>
       </c>
       <c r="E143" s="393"/>
@@ -65030,7 +65061,7 @@
       <c r="C145" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="D145" s="446" t="s">
+      <c r="D145" s="452" t="s">
         <v>727</v>
       </c>
       <c r="E145" s="393"/>
@@ -65154,7 +65185,7 @@
       <c r="C151" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="D151" s="446"/>
+      <c r="D151" s="452"/>
       <c r="E151" s="393"/>
       <c r="F151" s="2"/>
       <c r="G151" s="2"/>
@@ -65169,7 +65200,7 @@
       </c>
       <c r="B152" s="7"/>
       <c r="C152" s="71"/>
-      <c r="D152" s="446"/>
+      <c r="D152" s="452"/>
       <c r="E152" s="393"/>
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
@@ -65184,7 +65215,7 @@
       </c>
       <c r="B153" s="71"/>
       <c r="C153" s="71"/>
-      <c r="D153" s="446"/>
+      <c r="D153" s="452"/>
       <c r="E153" s="393"/>
       <c r="F153" s="2"/>
       <c r="G153" s="2"/>
@@ -65214,7 +65245,7 @@
       </c>
       <c r="B155" s="334"/>
       <c r="C155" s="71"/>
-      <c r="D155" s="446"/>
+      <c r="D155" s="452"/>
       <c r="E155" s="393"/>
       <c r="F155" s="2"/>
       <c r="G155" s="2"/>
@@ -65229,7 +65260,7 @@
       </c>
       <c r="B156" s="334"/>
       <c r="C156" s="71"/>
-      <c r="D156" s="446"/>
+      <c r="D156" s="452"/>
       <c r="E156" s="393"/>
       <c r="F156" s="2"/>
       <c r="G156" s="2"/>
@@ -65244,7 +65275,7 @@
       </c>
       <c r="B157" s="7"/>
       <c r="C157" s="333"/>
-      <c r="D157" s="446"/>
+      <c r="D157" s="452"/>
       <c r="E157" s="393"/>
       <c r="F157" s="2"/>
       <c r="G157" s="2"/>
@@ -65259,7 +65290,7 @@
       </c>
       <c r="B158" s="334"/>
       <c r="C158" s="71"/>
-      <c r="D158" s="446"/>
+      <c r="D158" s="452"/>
       <c r="E158" s="393"/>
       <c r="F158" s="2"/>
       <c r="G158" s="2"/>
@@ -76216,11 +76247,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A36:K36"/>
-    <mergeCell ref="A54:K54"/>
-    <mergeCell ref="A87:K87"/>
-    <mergeCell ref="A121:K121"/>
     <mergeCell ref="A141:F141"/>
     <mergeCell ref="D143:E143"/>
     <mergeCell ref="D157:E157"/>
@@ -76232,6 +76258,11 @@
     <mergeCell ref="D154:E154"/>
     <mergeCell ref="D155:E155"/>
     <mergeCell ref="D156:E156"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A54:K54"/>
+    <mergeCell ref="A87:K87"/>
+    <mergeCell ref="A121:K121"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>